<commit_message>
AW4 shield: R14 220R -> 2k2 (opto/base current limit), design review notes
With a high-CTR PC817 the relay driver could push ~50 mA through R14 (0.55 W
in a 0.25 W resistor). 2k2 limits base current to ~5 mA, still enough for
the 90 mA relay coils with BC337.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QHDQqfFe1juWLgZ1EWa6E5
</commit_message>
<xml_diff>
--- a/aw4_shield/bom_objednavka.xlsx
+++ b/aw4_shield/bom_objednavka.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Osazení" sheetId="2" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Objednávka!$A$5:$I$44</definedName>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Objednávka!$A$5:$I$43</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -58,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="558" uniqueCount="286">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="553" uniqueCount="285">
   <si>
     <t xml:space="preserve">AW4 shield v0.3 (THT, 100×100 mm) – seznam součástek k objednání</t>
   </si>
@@ -123,505 +123,502 @@
     <t xml:space="preserve">R11 R12</t>
   </si>
   <si>
-    <t xml:space="preserve">Rezistor 220 Ω</t>
+    <t xml:space="preserve">Rezistor 330 Ω</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0,25 W, 1 %, metalizovaný, DIN 0207 (montáž nastojato, rozteč 2,54)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R13 R17 R20 R23</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rezistor 1 kΩ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R3 R5 R7 R9 R18 R21 R24</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rezistor 2,2 kΩ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R14 R16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rezistor 10 kΩ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R4 R6 R8 R10 R15 R19 R22 R25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rezistor 100 kΩ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Diody</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dioda 1N4007</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 A / 1000 V, DO-41 – flyback solenoidů</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1N4007</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D12 D14 D16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dioda 1N4148</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DO-35</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1N4148</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Transil (TVS) 27 V</t>
+  </si>
+  <si>
+    <t xml:space="preserve">600 W, jednosměrný, DO-15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P6KE27A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zenerova dioda 12 V</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0,5 W, DO-35</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BZX55C12 (nebo BZX79C12)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zenerova dioda 15 V</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BZX55C15 (nebo BZX79C15)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D11 D13 D15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zenerova dioda 5,6 V</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0,5 W, DO-35 – ochrana vstupů</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BZX55C5V6 (nebo BZX79C5V6)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D3 D4 D5 D6 D7 D8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kondenzátory</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Elektrolyt 10 µF / 25 V</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ø5 mm, rozteč 2,0 mm, 105 °C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Elektrolyt 100 µF / 10 V (i 16 V)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ø6,3 mm, rozteč 2,5 mm, 105 °C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Elektrolyt 47 µF / 10 V (i 16 V)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Elektrolyt 470 µF / 25 V</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ø10 mm, rozteč 5 mm, 105 °C, low-ESR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">např. Panasonic řada FR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Feritová perla</t>
+  </si>
+  <si>
+    <t xml:space="preserve">axiální, ≥ 600 Ω @ 100 MHz, ≥ 1 A (montáž nastojato)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">např. Fair-Rite 2743019447</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L1 L2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kondenzátor 100 nF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">keramický, 50 V, X7R, rozteč 2,54 mm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">např. KEMET C320C104K5R5TA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C2 C5 C6 C7 C8 C10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Polovodiče</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LED zelená 3 mm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">indikace READY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">libovolná 3 mm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Optočlen PC817</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DIP-4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PC817C (Sharp / Everlight / Lite-On)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">U3 U4 U5 U6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P-MOSFET IRF4905</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TO-220 – ochrana proti přepólování</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IRF4905PBF (Infineon)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Q1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P-MOSFET IRF9540N</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TO-220 – spínání solenoidů</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IRF9540NPBF (Infineon)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Q3 Q4 Q5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spínaný stabilizátor 5 V / 1 A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">formát 7805 (SIP-3), vstup 6,5–36 V</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Traco TSR 1-2450</t>
+  </si>
+  <si>
+    <t xml:space="preserve">U1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tranzistor NPN BC337</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TO-92, pinout C-B-E (pad 1 = C)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BC337-40</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Q2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mechanické</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Distanční sloupek M3 + šroub</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pro 4 díry M3 v rozích</t>
+  </si>
+  <si>
+    <t xml:space="preserve">libovolné, např. 10 mm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">H1–H4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Patice pro pojistku TR5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rozteč 5,08 mm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Littelfuse 560 (TR5 patice)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pojistka TR5 5 A, pomalá (T)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TR5, rozteč 5,08 mm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Littelfuse řada 372, 5 A T</t>
+  </si>
+  <si>
+    <t xml:space="preserve">do F1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Relé 12 V SPDT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">kontakty 10 A, cívka 12 V</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Omron G5LE-1 DC12 (pinově kompatibilní: Songle SRD-12VDC-SL-C)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">K1 K2 K3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Konektory</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dutinková lišta 1×15 (patice pro Nano)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rozteč 2,54 mm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">libovolná</t>
+  </si>
+  <si>
+    <t xml:space="preserve">U2 (patice)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kabelová část JST-XH 4 pin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pouzdro + 4 kontakty</t>
+  </si>
+  <si>
+    <t xml:space="preserve">JST XHP-4 + 4× SXH-001T-P0.6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">kabel k displeji</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kolíková lišta 1×2 + jumper</t>
+  </si>
+  <si>
+    <t xml:space="preserve">libovolná + zkratovací propojka 2,54</t>
+  </si>
+  <si>
+    <t xml:space="preserve">JP1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kolíková lišta 1×7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rozteč 2,54 mm (volitelné – rezerva)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">libovolná (odlomit z 1×40)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Konektor JST-XH 4 pin (do DPS)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rozteč 2,5 mm, vertikální</t>
+  </si>
+  <si>
+    <t xml:space="preserve">JST B4B-XH-A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Svorkovnice 2 pól</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rozteč 5,08 mm, do DPS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Phoenix Contact MKDS 1,5/2-5,08 (1715721)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Svorkovnice 6 pól</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Phoenix Contact MKDS 1,5/6-5,08 (1715763)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J2 J3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Moduly</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Arduino Nano (ATmega328P, 5 V)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">zasouvá se do patic (viz níže)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Arduino Nano nebo klon s CH340</t>
+  </si>
+  <si>
+    <t xml:space="preserve">U2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Displej Nextion 2,4″</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UART, 5 V</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nextion NX3224T024 (nebo NX4024T032 3,2″)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mimo desku, přes J5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Celkem kusů k objednání:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Součástek osazených na desce (referencí ve schématu): 74</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Postup osazení – od nejnižších součástek po nejvyšší</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Na desce je na potisku vytištěné, co kam patří (sloupec 'Na potisku'). Označení (R18 …) je v osazovacím výkresu docs/aw4_shield_osazovaci_vykres.pdf a v interaktivním BOM.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Krok</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Označení</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Na potisku</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hodnota ve schématu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pozor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Osazeno ✓</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. rezistory</t>
+  </si>
+  <si>
+    <t xml:space="preserve">100k</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0R</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1k</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10k</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">100R</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">330</t>
   </si>
   <si>
     <t xml:space="preserve">R14</t>
   </si>
   <si>
-    <t xml:space="preserve">Rezistor 330 Ω</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0,25 W, 1 %, metalizovaný, DIN 0207 (montáž nastojato, rozteč 2,54)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R13 R17 R20 R23</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rezistor 1 kΩ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R3 R5 R7 R9 R18 R21 R24</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rezistor 2,2 kΩ</t>
+    <t xml:space="preserve">2k2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R15</t>
   </si>
   <si>
     <t xml:space="preserve">R16</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rezistor 10 kΩ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R4 R6 R8 R10 R15 R19 R22 R25</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rezistor 100 kΩ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Diody</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dioda 1N4007</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1 A / 1000 V, DO-41 – flyback solenoidů</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1N4007</t>
-  </si>
-  <si>
-    <t xml:space="preserve">D12 D14 D16</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dioda 1N4148</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DO-35</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1N4148</t>
-  </si>
-  <si>
-    <t xml:space="preserve">D9</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Transil (TVS) 27 V</t>
-  </si>
-  <si>
-    <t xml:space="preserve">600 W, jednosměrný, DO-15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P6KE27A</t>
-  </si>
-  <si>
-    <t xml:space="preserve">D2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Zenerova dioda 12 V</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0,5 W, DO-35</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BZX55C12 (nebo BZX79C12)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">D1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Zenerova dioda 15 V</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BZX55C15 (nebo BZX79C15)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">D11 D13 D15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Zenerova dioda 5,6 V</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0,5 W, DO-35 – ochrana vstupů</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BZX55C5V6 (nebo BZX79C5V6)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">D3 D4 D5 D6 D7 D8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kondenzátory</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Elektrolyt 10 µF / 25 V</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ø5 mm, rozteč 2,0 mm, 105 °C</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Elektrolyt 100 µF / 10 V (i 16 V)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ø6,3 mm, rozteč 2,5 mm, 105 °C</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C9</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Elektrolyt 47 µF / 10 V (i 16 V)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Elektrolyt 470 µF / 25 V</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ø10 mm, rozteč 5 mm, 105 °C, low-ESR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">např. Panasonic řada FR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Feritová perla</t>
-  </si>
-  <si>
-    <t xml:space="preserve">axiální, ≥ 600 Ω @ 100 MHz, ≥ 1 A (montáž nastojato)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">např. Fair-Rite 2743019447</t>
-  </si>
-  <si>
-    <t xml:space="preserve">L1 L2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kondenzátor 100 nF</t>
-  </si>
-  <si>
-    <t xml:space="preserve">keramický, 50 V, X7R, rozteč 2,54 mm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">např. KEMET C320C104K5R5TA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C2 C5 C6 C7 C8 C10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Polovodiče</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LED zelená 3 mm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">indikace READY</t>
-  </si>
-  <si>
-    <t xml:space="preserve">libovolná 3 mm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">D10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Optočlen PC817</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DIP-4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PC817C (Sharp / Everlight / Lite-On)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">U3 U4 U5 U6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P-MOSFET IRF4905</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TO-220 – ochrana proti přepólování</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IRF4905PBF (Infineon)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Q1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P-MOSFET IRF9540N</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TO-220 – spínání solenoidů</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IRF9540NPBF (Infineon)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Q3 Q4 Q5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Spínaný stabilizátor 5 V / 1 A</t>
-  </si>
-  <si>
-    <t xml:space="preserve">formát 7805 (SIP-3), vstup 6,5–36 V</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Traco TSR 1-2450</t>
-  </si>
-  <si>
-    <t xml:space="preserve">U1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tranzistor NPN BC337</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TO-92, pinout C-B-E (pad 1 = C)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BC337-40</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Q2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mechanické</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Distanční sloupek M3 + šroub</t>
-  </si>
-  <si>
-    <t xml:space="preserve">pro 4 díry M3 v rozích</t>
-  </si>
-  <si>
-    <t xml:space="preserve">libovolné, např. 10 mm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">H1–H4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Patice pro pojistku TR5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rozteč 5,08 mm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Littelfuse 560 (TR5 patice)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pojistka TR5 5 A, pomalá (T)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TR5, rozteč 5,08 mm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Littelfuse řada 372, 5 A T</t>
-  </si>
-  <si>
-    <t xml:space="preserve">do F1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Relé 12 V SPDT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">kontakty 10 A, cívka 12 V</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Omron G5LE-1 DC12 (pinově kompatibilní: Songle SRD-12VDC-SL-C)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">K1 K2 K3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Konektory</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dutinková lišta 1×15 (patice pro Nano)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rozteč 2,54 mm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">libovolná</t>
-  </si>
-  <si>
-    <t xml:space="preserve">U2 (patice)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kabelová část JST-XH 4 pin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">pouzdro + 4 kontakty</t>
-  </si>
-  <si>
-    <t xml:space="preserve">JST XHP-4 + 4× SXH-001T-P0.6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">kabel k displeji</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kolíková lišta 1×2 + jumper</t>
-  </si>
-  <si>
-    <t xml:space="preserve">libovolná + zkratovací propojka 2,54</t>
-  </si>
-  <si>
-    <t xml:space="preserve">JP1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kolíková lišta 1×7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rozteč 2,54 mm (volitelné – rezerva)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">libovolná (odlomit z 1×40)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">J6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Konektor JST-XH 4 pin (do DPS)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rozteč 2,5 mm, vertikální</t>
-  </si>
-  <si>
-    <t xml:space="preserve">JST B4B-XH-A</t>
-  </si>
-  <si>
-    <t xml:space="preserve">J5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Svorkovnice 2 pól</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rozteč 5,08 mm, do DPS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Phoenix Contact MKDS 1,5/2-5,08 (1715721)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">J1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Svorkovnice 6 pól</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Phoenix Contact MKDS 1,5/6-5,08 (1715763)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">J2 J3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Moduly</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Arduino Nano (ATmega328P, 5 V)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">zasouvá se do patic (viz níže)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Arduino Nano nebo klon s CH340</t>
-  </si>
-  <si>
-    <t xml:space="preserve">U2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Displej Nextion 2,4″</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UART, 5 V</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nextion NX3224T024 (nebo NX4024T032 3,2″)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">mimo desku, přes J5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Celkem kusů k objednání:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Součástek osazených na desce (referencí ve schématu): 74</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Postup osazení – od nejnižších součástek po nejvyšší</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Na desce je na potisku vytištěné, co kam patří (sloupec 'Na potisku'). Označení (R18 …) je v osazovacím výkresu docs/aw4_shield_osazovaci_vykres.pdf a v interaktivním BOM.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Krok</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Označení</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Na potisku</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hodnota ve schématu</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pozor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Osazeno ✓</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. rezistory</t>
-  </si>
-  <si>
-    <t xml:space="preserve">100k</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0R</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1k</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10k</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R9</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">100R</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R13</t>
-  </si>
-  <si>
-    <t xml:space="preserve">330</t>
-  </si>
-  <si>
-    <t xml:space="preserve">220</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2k2</t>
   </si>
   <si>
     <t xml:space="preserve">R17</t>
@@ -1480,7 +1477,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:I47"/>
+  <dimension ref="A1:I46"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
@@ -1603,7 +1600,7 @@
       </c>
       <c r="I7" s="10"/>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="n">
         <v>3</v>
       </c>
@@ -1614,24 +1611,24 @@
         <v>21</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="E8" s="7" t="s">
         <v>16</v>
       </c>
       <c r="F8" s="8" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G8" s="9" t="n">
         <f aca="false">F8*$C$2+IF(TRUE(),$G$2,0)</f>
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="H8" s="7" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="I8" s="7"/>
     </row>
-    <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="10" t="n">
         <v>4</v>
       </c>
@@ -1639,20 +1636,20 @@
         <v>13</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D9" s="10" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="E9" s="10" t="s">
         <v>16</v>
       </c>
       <c r="F9" s="11" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="G9" s="12" t="n">
         <f aca="false">F9*$C$2+IF(TRUE(),$G$2,0)</f>
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="H9" s="10" t="s">
         <v>25</v>
@@ -1676,11 +1673,11 @@
         <v>16</v>
       </c>
       <c r="F10" s="8" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="G10" s="9" t="n">
         <f aca="false">F10*$C$2+IF(TRUE(),$G$2,0)</f>
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="H10" s="7" t="s">
         <v>27</v>
@@ -1704,11 +1701,11 @@
         <v>16</v>
       </c>
       <c r="F11" s="11" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="G11" s="12" t="n">
         <f aca="false">F11*$C$2+IF(TRUE(),$G$2,0)</f>
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="H11" s="10" t="s">
         <v>29</v>
@@ -1732,11 +1729,11 @@
         <v>16</v>
       </c>
       <c r="F12" s="8" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="G12" s="9" t="n">
         <f aca="false">F12*$C$2+IF(TRUE(),$G$2,0)</f>
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="H12" s="7" t="s">
         <v>31</v>
@@ -1748,26 +1745,26 @@
         <v>8</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D13" s="10" t="s">
-        <v>19</v>
+        <v>34</v>
       </c>
       <c r="E13" s="10" t="s">
-        <v>16</v>
+        <v>35</v>
       </c>
       <c r="F13" s="11" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G13" s="12" t="n">
         <f aca="false">F13*$C$2+IF(TRUE(),$G$2,0)</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H13" s="10" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="I13" s="10"/>
     </row>
@@ -1776,26 +1773,26 @@
         <v>9</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D14" s="7" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E14" s="7" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="F14" s="8" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G14" s="9" t="n">
         <f aca="false">F14*$C$2+IF(TRUE(),$G$2,0)</f>
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H14" s="7" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="I14" s="7"/>
     </row>
@@ -1804,16 +1801,16 @@
         <v>10</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D15" s="10" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E15" s="10" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="F15" s="11" t="n">
         <v>1</v>
@@ -1823,7 +1820,7 @@
         <v>3</v>
       </c>
       <c r="H15" s="10" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="I15" s="10"/>
     </row>
@@ -1832,16 +1829,16 @@
         <v>11</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="E16" s="7" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F16" s="8" t="n">
         <v>1</v>
@@ -1851,7 +1848,7 @@
         <v>3</v>
       </c>
       <c r="H16" s="7" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="I16" s="7"/>
     </row>
@@ -1860,26 +1857,26 @@
         <v>12</v>
       </c>
       <c r="B17" s="10" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C17" s="10" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D17" s="10" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="E17" s="10" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F17" s="11" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G17" s="12" t="n">
         <f aca="false">F17*$C$2+IF(TRUE(),$G$2,0)</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H17" s="10" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="I17" s="10"/>
     </row>
@@ -1888,26 +1885,26 @@
         <v>13</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D18" s="7" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="E18" s="7" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="F18" s="8" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G18" s="9" t="n">
         <f aca="false">F18*$C$2+IF(TRUE(),$G$2,0)</f>
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="H18" s="7" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="I18" s="7"/>
     </row>
@@ -1916,26 +1913,26 @@
         <v>14</v>
       </c>
       <c r="B19" s="10" t="s">
-        <v>34</v>
+        <v>56</v>
       </c>
       <c r="C19" s="10" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="D19" s="10" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="E19" s="10" t="s">
-        <v>56</v>
+        <v>16</v>
       </c>
       <c r="F19" s="11" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="G19" s="12" t="n">
         <f aca="false">F19*$C$2+IF(TRUE(),$G$2,0)</f>
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="H19" s="10" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="I19" s="10"/>
     </row>
@@ -1944,13 +1941,13 @@
         <v>15</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D20" s="7" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E20" s="7" t="s">
         <v>16</v>
@@ -1963,7 +1960,7 @@
         <v>3</v>
       </c>
       <c r="H20" s="7" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="I20" s="7"/>
     </row>
@@ -1972,13 +1969,13 @@
         <v>16</v>
       </c>
       <c r="B21" s="10" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="C21" s="10" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D21" s="10" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="E21" s="10" t="s">
         <v>16</v>
@@ -2000,16 +1997,16 @@
         <v>17</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="C22" s="7" t="s">
         <v>65</v>
       </c>
       <c r="D22" s="7" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="E22" s="7" t="s">
-        <v>16</v>
+        <v>67</v>
       </c>
       <c r="F22" s="8" t="n">
         <v>1</v>
@@ -2019,63 +2016,63 @@
         <v>3</v>
       </c>
       <c r="H22" s="7" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="I22" s="7"/>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="10" t="n">
         <v>18</v>
       </c>
       <c r="B23" s="10" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="C23" s="10" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D23" s="10" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="E23" s="10" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F23" s="11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G23" s="12" t="n">
         <f aca="false">F23*$C$2+IF(TRUE(),$G$2,0)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H23" s="10" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="I23" s="10"/>
     </row>
-    <row r="24" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="7" t="n">
         <v>19</v>
       </c>
       <c r="B24" s="7" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="C24" s="7" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D24" s="7" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="E24" s="7" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="F24" s="8" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="G24" s="9" t="n">
         <f aca="false">F24*$C$2+IF(TRUE(),$G$2,0)</f>
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="H24" s="7" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="I24" s="7"/>
     </row>
@@ -2084,26 +2081,26 @@
         <v>20</v>
       </c>
       <c r="B25" s="10" t="s">
-        <v>58</v>
+        <v>77</v>
       </c>
       <c r="C25" s="10" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="D25" s="10" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="E25" s="10" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="F25" s="11" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="G25" s="12" t="n">
-        <f aca="false">F25*$C$2+IF(TRUE(),$G$2,0)</f>
-        <v>8</v>
+        <f aca="false">F25*$C$2</f>
+        <v>1</v>
       </c>
       <c r="H25" s="10" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="I25" s="10"/>
     </row>
@@ -2112,26 +2109,26 @@
         <v>21</v>
       </c>
       <c r="B26" s="7" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C26" s="7" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="D26" s="7" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="E26" s="7" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="F26" s="8" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G26" s="9" t="n">
         <f aca="false">F26*$C$2</f>
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H26" s="7" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="I26" s="7"/>
     </row>
@@ -2140,26 +2137,26 @@
         <v>22</v>
       </c>
       <c r="B27" s="10" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C27" s="10" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D27" s="10" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="E27" s="10" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="F27" s="11" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G27" s="12" t="n">
         <f aca="false">F27*$C$2</f>
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H27" s="10" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="I27" s="10"/>
     </row>
@@ -2168,26 +2165,26 @@
         <v>23</v>
       </c>
       <c r="B28" s="7" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C28" s="7" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="D28" s="7" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="E28" s="7" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="F28" s="8" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G28" s="9" t="n">
         <f aca="false">F28*$C$2</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H28" s="7" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="I28" s="7"/>
     </row>
@@ -2196,26 +2193,26 @@
         <v>24</v>
       </c>
       <c r="B29" s="10" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C29" s="10" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="D29" s="10" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="E29" s="10" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="F29" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G29" s="12" t="n">
         <f aca="false">F29*$C$2</f>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H29" s="10" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="I29" s="10"/>
     </row>
@@ -2224,16 +2221,16 @@
         <v>25</v>
       </c>
       <c r="B30" s="7" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C30" s="7" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D30" s="7" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="E30" s="7" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="F30" s="8" t="n">
         <v>1</v>
@@ -2243,7 +2240,7 @@
         <v>1</v>
       </c>
       <c r="H30" s="7" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="I30" s="7"/>
     </row>
@@ -2252,26 +2249,26 @@
         <v>26</v>
       </c>
       <c r="B31" s="10" t="s">
-        <v>79</v>
+        <v>102</v>
       </c>
       <c r="C31" s="10" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="D31" s="10" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="E31" s="10" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="F31" s="11" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G31" s="12" t="n">
         <f aca="false">F31*$C$2</f>
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H31" s="10" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="I31" s="10"/>
     </row>
@@ -2280,26 +2277,26 @@
         <v>27</v>
       </c>
       <c r="B32" s="7" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="C32" s="7" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="D32" s="7" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="E32" s="7" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="F32" s="8" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G32" s="9" t="n">
         <f aca="false">F32*$C$2</f>
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H32" s="7" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="I32" s="7"/>
     </row>
@@ -2308,16 +2305,16 @@
         <v>28</v>
       </c>
       <c r="B33" s="10" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="C33" s="10" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="D33" s="10" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E33" s="10" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="F33" s="11" t="n">
         <v>1</v>
@@ -2327,35 +2324,35 @@
         <v>1</v>
       </c>
       <c r="H33" s="10" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="I33" s="10"/>
     </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="34" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="7" t="n">
         <v>29</v>
       </c>
       <c r="B34" s="7" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="C34" s="7" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D34" s="7" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="E34" s="7" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="F34" s="8" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G34" s="9" t="n">
         <f aca="false">F34*$C$2</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H34" s="7" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="I34" s="7"/>
     </row>
@@ -2364,54 +2361,54 @@
         <v>30</v>
       </c>
       <c r="B35" s="10" t="s">
-        <v>104</v>
+        <v>119</v>
       </c>
       <c r="C35" s="10" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="D35" s="10" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="E35" s="10" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="F35" s="11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G35" s="12" t="n">
         <f aca="false">F35*$C$2</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H35" s="10" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="I35" s="10"/>
     </row>
-    <row r="36" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="7" t="n">
         <v>31</v>
       </c>
       <c r="B36" s="7" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="C36" s="7" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="D36" s="7" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="E36" s="7" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="F36" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G36" s="9" t="n">
         <f aca="false">F36*$C$2</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H36" s="7" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="I36" s="7"/>
     </row>
@@ -2420,16 +2417,16 @@
         <v>32</v>
       </c>
       <c r="B37" s="10" t="s">
+        <v>119</v>
+      </c>
+      <c r="C37" s="10" t="s">
+        <v>128</v>
+      </c>
+      <c r="D37" s="10" t="s">
         <v>121</v>
       </c>
-      <c r="C37" s="10" t="s">
-        <v>126</v>
-      </c>
-      <c r="D37" s="10" t="s">
-        <v>127</v>
-      </c>
       <c r="E37" s="10" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="F37" s="11" t="n">
         <v>1</v>
@@ -2439,7 +2436,7 @@
         <v>1</v>
       </c>
       <c r="H37" s="10" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="I37" s="10"/>
     </row>
@@ -2448,16 +2445,16 @@
         <v>33</v>
       </c>
       <c r="B38" s="7" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="C38" s="7" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D38" s="7" t="s">
-        <v>123</v>
+        <v>132</v>
       </c>
       <c r="E38" s="7" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="F38" s="8" t="n">
         <v>1</v>
@@ -2467,7 +2464,7 @@
         <v>1</v>
       </c>
       <c r="H38" s="7" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="I38" s="7"/>
     </row>
@@ -2476,16 +2473,16 @@
         <v>34</v>
       </c>
       <c r="B39" s="10" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="C39" s="10" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="D39" s="10" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="E39" s="10" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="F39" s="11" t="n">
         <v>1</v>
@@ -2495,7 +2492,7 @@
         <v>1</v>
       </c>
       <c r="H39" s="10" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="I39" s="10"/>
     </row>
@@ -2504,16 +2501,16 @@
         <v>35</v>
       </c>
       <c r="B40" s="7" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="C40" s="7" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="D40" s="7" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="E40" s="7" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="F40" s="8" t="n">
         <v>1</v>
@@ -2523,7 +2520,7 @@
         <v>1</v>
       </c>
       <c r="H40" s="7" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="I40" s="7"/>
     </row>
@@ -2532,26 +2529,26 @@
         <v>36</v>
       </c>
       <c r="B41" s="10" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="C41" s="10" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="D41" s="10" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="E41" s="10" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="F41" s="11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G41" s="12" t="n">
         <f aca="false">F41*$C$2</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H41" s="10" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="I41" s="10"/>
     </row>
@@ -2560,26 +2557,26 @@
         <v>37</v>
       </c>
       <c r="B42" s="7" t="s">
-        <v>121</v>
+        <v>146</v>
       </c>
       <c r="C42" s="7" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="D42" s="7" t="s">
-        <v>142</v>
+        <v>148</v>
       </c>
       <c r="E42" s="7" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="F42" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G42" s="9" t="n">
         <f aca="false">F42*$C$2</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H42" s="7" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="I42" s="7"/>
     </row>
@@ -2588,16 +2585,16 @@
         <v>38</v>
       </c>
       <c r="B43" s="10" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="C43" s="10" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="D43" s="10" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="E43" s="10" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="F43" s="11" t="n">
         <v>1</v>
@@ -2607,54 +2604,26 @@
         <v>1</v>
       </c>
       <c r="H43" s="10" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="I43" s="10"/>
     </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="7" t="n">
-        <v>39</v>
-      </c>
-      <c r="B44" s="7" t="s">
-        <v>148</v>
-      </c>
-      <c r="C44" s="7" t="s">
-        <v>153</v>
-      </c>
-      <c r="D44" s="7" t="s">
-        <v>154</v>
-      </c>
-      <c r="E44" s="7" t="s">
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E45" s="2" t="s">
         <v>155</v>
       </c>
-      <c r="F44" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="G44" s="9" t="n">
-        <f aca="false">F44*$C$2</f>
-        <v>1</v>
-      </c>
-      <c r="H44" s="7" t="s">
+      <c r="G45" s="2" t="n">
+        <f aca="false">SUM(G6:G43)</f>
+        <v>121</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E46" s="13" t="s">
         <v>156</v>
       </c>
-      <c r="I44" s="7"/>
-    </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E46" s="2" t="s">
-        <v>157</v>
-      </c>
-      <c r="G46" s="2" t="n">
-        <f aca="false">SUM(G6:G44)</f>
-        <v>123</v>
-      </c>
-    </row>
-    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E47" s="13" t="s">
-        <v>158</v>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A5:I44"/>
+  <autoFilter ref="A5:I43"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -2686,40 +2655,40 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
+        <v>159</v>
+      </c>
+      <c r="B4" s="14" t="s">
+        <v>160</v>
+      </c>
+      <c r="C4" s="14" t="s">
         <v>161</v>
-      </c>
-      <c r="B4" s="14" t="s">
-        <v>162</v>
-      </c>
-      <c r="C4" s="14" t="s">
-        <v>163</v>
       </c>
       <c r="D4" s="14" t="s">
         <v>6</v>
       </c>
       <c r="E4" s="14" t="s">
+        <v>162</v>
+      </c>
+      <c r="F4" s="14" t="s">
+        <v>163</v>
+      </c>
+      <c r="G4" s="14" t="s">
         <v>164</v>
-      </c>
-      <c r="F4" s="14" t="s">
-        <v>165</v>
-      </c>
-      <c r="G4" s="14" t="s">
-        <v>166</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="15" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="B5" s="16"/>
       <c r="C5" s="16"/>
@@ -2731,16 +2700,16 @@
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="17"/>
       <c r="B6" s="17" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C6" s="17" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="D6" s="17" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="E6" s="17" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="F6" s="17"/>
       <c r="G6" s="17"/>
@@ -2751,13 +2720,13 @@
         <v>17</v>
       </c>
       <c r="C7" s="17" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="D7" s="17" t="s">
         <v>14</v>
       </c>
       <c r="E7" s="17" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="F7" s="17"/>
       <c r="G7" s="17"/>
@@ -2765,16 +2734,16 @@
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="17"/>
       <c r="B8" s="17" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="C8" s="17" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="D8" s="17" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="E8" s="17" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="F8" s="17"/>
       <c r="G8" s="17"/>
@@ -2782,16 +2751,16 @@
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="17"/>
       <c r="B9" s="17" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="C9" s="17" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="D9" s="17" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="E9" s="17" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="F9" s="17"/>
       <c r="G9" s="17"/>
@@ -2799,16 +2768,16 @@
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="17"/>
       <c r="B10" s="17" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="C10" s="17" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="D10" s="17" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="E10" s="17" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="F10" s="17"/>
       <c r="G10" s="17"/>
@@ -2816,16 +2785,16 @@
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="17"/>
       <c r="B11" s="17" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="C11" s="17" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="D11" s="17" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="E11" s="17" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="F11" s="17"/>
       <c r="G11" s="17"/>
@@ -2833,16 +2802,16 @@
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="17"/>
       <c r="B12" s="17" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="C12" s="17" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="D12" s="17" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="E12" s="17" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="F12" s="17"/>
       <c r="G12" s="17"/>
@@ -2850,16 +2819,16 @@
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="17"/>
       <c r="B13" s="17" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="C13" s="17" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="D13" s="17" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="E13" s="17" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="F13" s="17"/>
       <c r="G13" s="17"/>
@@ -2867,16 +2836,16 @@
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="17"/>
       <c r="B14" s="17" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="C14" s="17" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="D14" s="17" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="E14" s="17" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="F14" s="17"/>
       <c r="G14" s="17"/>
@@ -2884,16 +2853,16 @@
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="17"/>
       <c r="B15" s="17" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="C15" s="17" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="D15" s="17" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="E15" s="17" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="F15" s="17"/>
       <c r="G15" s="17"/>
@@ -2901,16 +2870,16 @@
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="17"/>
       <c r="B16" s="17" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="C16" s="17" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="D16" s="17" t="s">
         <v>18</v>
       </c>
       <c r="E16" s="17" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="F16" s="17"/>
       <c r="G16" s="17"/>
@@ -2918,16 +2887,16 @@
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="17"/>
       <c r="B17" s="17" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="C17" s="17" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="D17" s="17" t="s">
         <v>18</v>
       </c>
       <c r="E17" s="17" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="F17" s="17"/>
       <c r="G17" s="17"/>
@@ -2935,16 +2904,16 @@
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="17"/>
       <c r="B18" s="17" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="C18" s="17" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="D18" s="17" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="E18" s="17" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="F18" s="17"/>
       <c r="G18" s="17"/>
@@ -2952,16 +2921,16 @@
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="17"/>
       <c r="B19" s="17" t="s">
-        <v>22</v>
+        <v>183</v>
       </c>
       <c r="C19" s="17" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="D19" s="17" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="E19" s="17" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F19" s="17"/>
       <c r="G19" s="17"/>
@@ -2969,16 +2938,16 @@
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="17"/>
       <c r="B20" s="17" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="C20" s="17" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="D20" s="17" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="E20" s="17" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="F20" s="17"/>
       <c r="G20" s="17"/>
@@ -2986,16 +2955,16 @@
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="17"/>
       <c r="B21" s="17" t="s">
-        <v>29</v>
+        <v>186</v>
       </c>
       <c r="C21" s="17" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="D21" s="17" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E21" s="17" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="F21" s="17"/>
       <c r="G21" s="17"/>
@@ -3003,16 +2972,16 @@
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="17"/>
       <c r="B22" s="17" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C22" s="17" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="D22" s="17" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="E22" s="17" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="F22" s="17"/>
       <c r="G22" s="17"/>
@@ -3020,16 +2989,16 @@
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="17"/>
       <c r="B23" s="17" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="C23" s="17" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="D23" s="17" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="E23" s="17" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="F23" s="17"/>
       <c r="G23" s="17"/>
@@ -3037,16 +3006,16 @@
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="17"/>
       <c r="B24" s="17" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C24" s="17" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="D24" s="17" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="E24" s="17" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="F24" s="17"/>
       <c r="G24" s="17"/>
@@ -3054,16 +3023,16 @@
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="17"/>
       <c r="B25" s="17" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C25" s="17" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="D25" s="17" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="E25" s="17" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="F25" s="17"/>
       <c r="G25" s="17"/>
@@ -3071,16 +3040,16 @@
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="17"/>
       <c r="B26" s="17" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="C26" s="17" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="D26" s="17" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="E26" s="17" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="F26" s="17"/>
       <c r="G26" s="17"/>
@@ -3088,16 +3057,16 @@
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="17"/>
       <c r="B27" s="17" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="C27" s="17" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="D27" s="17" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="E27" s="17" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="F27" s="17"/>
       <c r="G27" s="17"/>
@@ -3105,16 +3074,16 @@
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="17"/>
       <c r="B28" s="17" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="C28" s="17" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="D28" s="17" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="E28" s="17" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="F28" s="17"/>
       <c r="G28" s="17"/>
@@ -3122,16 +3091,16 @@
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="17"/>
       <c r="B29" s="17" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="C29" s="17" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="D29" s="17" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="E29" s="17" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="F29" s="17"/>
       <c r="G29" s="17"/>
@@ -3139,23 +3108,23 @@
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="17"/>
       <c r="B30" s="17" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="C30" s="17" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="D30" s="17" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="E30" s="17" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="F30" s="17"/>
       <c r="G30" s="17"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="15" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B31" s="16"/>
       <c r="C31" s="16"/>
@@ -3167,291 +3136,291 @@
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="17"/>
       <c r="B32" s="17" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C32" s="17" t="s">
+        <v>197</v>
+      </c>
+      <c r="D32" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="E32" s="17" t="s">
         <v>198</v>
       </c>
-      <c r="D32" s="17" t="s">
-        <v>47</v>
-      </c>
-      <c r="E32" s="17" t="s">
+      <c r="F32" s="18" t="s">
         <v>199</v>
-      </c>
-      <c r="F32" s="18" t="s">
-        <v>200</v>
       </c>
       <c r="G32" s="17"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="17"/>
       <c r="B33" s="17" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C33" s="17" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="D33" s="17" t="s">
+        <v>41</v>
+      </c>
+      <c r="E33" s="17" t="s">
         <v>43</v>
       </c>
-      <c r="E33" s="17" t="s">
-        <v>45</v>
-      </c>
       <c r="F33" s="18" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="G33" s="17"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="17"/>
       <c r="B34" s="17" t="s">
+        <v>201</v>
+      </c>
+      <c r="C34" s="17" t="s">
         <v>202</v>
       </c>
-      <c r="C34" s="17" t="s">
+      <c r="D34" s="17" t="s">
+        <v>52</v>
+      </c>
+      <c r="E34" s="17" t="s">
         <v>203</v>
       </c>
-      <c r="D34" s="17" t="s">
-        <v>54</v>
-      </c>
-      <c r="E34" s="17" t="s">
-        <v>204</v>
-      </c>
       <c r="F34" s="18" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="G34" s="17"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="17"/>
       <c r="B35" s="17" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="C35" s="17" t="s">
+        <v>202</v>
+      </c>
+      <c r="D35" s="17" t="s">
+        <v>52</v>
+      </c>
+      <c r="E35" s="17" t="s">
         <v>203</v>
       </c>
-      <c r="D35" s="17" t="s">
-        <v>54</v>
-      </c>
-      <c r="E35" s="17" t="s">
-        <v>204</v>
-      </c>
       <c r="F35" s="18" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="G35" s="17"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="17"/>
       <c r="B36" s="17" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="C36" s="17" t="s">
+        <v>202</v>
+      </c>
+      <c r="D36" s="17" t="s">
+        <v>52</v>
+      </c>
+      <c r="E36" s="17" t="s">
         <v>203</v>
       </c>
-      <c r="D36" s="17" t="s">
-        <v>54</v>
-      </c>
-      <c r="E36" s="17" t="s">
-        <v>204</v>
-      </c>
       <c r="F36" s="18" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="G36" s="17"/>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="17"/>
       <c r="B37" s="17" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="C37" s="17" t="s">
+        <v>202</v>
+      </c>
+      <c r="D37" s="17" t="s">
+        <v>52</v>
+      </c>
+      <c r="E37" s="17" t="s">
         <v>203</v>
       </c>
-      <c r="D37" s="17" t="s">
-        <v>54</v>
-      </c>
-      <c r="E37" s="17" t="s">
-        <v>204</v>
-      </c>
       <c r="F37" s="18" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="G37" s="17"/>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="17"/>
       <c r="B38" s="17" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="C38" s="17" t="s">
+        <v>202</v>
+      </c>
+      <c r="D38" s="17" t="s">
+        <v>52</v>
+      </c>
+      <c r="E38" s="17" t="s">
         <v>203</v>
       </c>
-      <c r="D38" s="17" t="s">
-        <v>54</v>
-      </c>
-      <c r="E38" s="17" t="s">
-        <v>204</v>
-      </c>
       <c r="F38" s="18" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="G38" s="17"/>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="17"/>
       <c r="B39" s="17" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C39" s="17" t="s">
+        <v>202</v>
+      </c>
+      <c r="D39" s="17" t="s">
+        <v>52</v>
+      </c>
+      <c r="E39" s="17" t="s">
         <v>203</v>
       </c>
-      <c r="D39" s="17" t="s">
-        <v>54</v>
-      </c>
-      <c r="E39" s="17" t="s">
-        <v>204</v>
-      </c>
       <c r="F39" s="18" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="G39" s="17"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="17"/>
       <c r="B40" s="17" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C40" s="17" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="D40" s="17" t="s">
+        <v>37</v>
+      </c>
+      <c r="E40" s="17" t="s">
         <v>39</v>
       </c>
-      <c r="E40" s="17" t="s">
-        <v>41</v>
-      </c>
       <c r="F40" s="18" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="G40" s="17"/>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="17"/>
       <c r="B41" s="17" t="s">
+        <v>210</v>
+      </c>
+      <c r="C41" s="17" t="s">
         <v>211</v>
       </c>
-      <c r="C41" s="17" t="s">
+      <c r="D41" s="17" t="s">
+        <v>49</v>
+      </c>
+      <c r="E41" s="17" t="s">
         <v>212</v>
       </c>
-      <c r="D41" s="17" t="s">
-        <v>51</v>
-      </c>
-      <c r="E41" s="17" t="s">
-        <v>213</v>
-      </c>
       <c r="F41" s="18" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="G41" s="17"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="17"/>
       <c r="B42" s="17" t="s">
+        <v>213</v>
+      </c>
+      <c r="C42" s="17" t="s">
         <v>214</v>
       </c>
-      <c r="C42" s="17" t="s">
-        <v>215</v>
-      </c>
       <c r="D42" s="17" t="s">
+        <v>33</v>
+      </c>
+      <c r="E42" s="17" t="s">
         <v>35</v>
       </c>
-      <c r="E42" s="17" t="s">
-        <v>37</v>
-      </c>
       <c r="F42" s="18" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="G42" s="17"/>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="17"/>
       <c r="B43" s="17" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C43" s="17" t="s">
+        <v>211</v>
+      </c>
+      <c r="D43" s="17" t="s">
+        <v>49</v>
+      </c>
+      <c r="E43" s="17" t="s">
         <v>212</v>
       </c>
-      <c r="D43" s="17" t="s">
-        <v>51</v>
-      </c>
-      <c r="E43" s="17" t="s">
-        <v>213</v>
-      </c>
       <c r="F43" s="18" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="G43" s="17"/>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="17"/>
       <c r="B44" s="17" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C44" s="17" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="D44" s="17" t="s">
+        <v>33</v>
+      </c>
+      <c r="E44" s="17" t="s">
         <v>35</v>
       </c>
-      <c r="E44" s="17" t="s">
-        <v>37</v>
-      </c>
       <c r="F44" s="18" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="G44" s="17"/>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="17"/>
       <c r="B45" s="17" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C45" s="17" t="s">
+        <v>211</v>
+      </c>
+      <c r="D45" s="17" t="s">
+        <v>49</v>
+      </c>
+      <c r="E45" s="17" t="s">
         <v>212</v>
       </c>
-      <c r="D45" s="17" t="s">
-        <v>51</v>
-      </c>
-      <c r="E45" s="17" t="s">
-        <v>213</v>
-      </c>
       <c r="F45" s="18" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="G45" s="17"/>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="17"/>
       <c r="B46" s="17" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="C46" s="17" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="D46" s="17" t="s">
+        <v>33</v>
+      </c>
+      <c r="E46" s="17" t="s">
         <v>35</v>
       </c>
-      <c r="E46" s="17" t="s">
-        <v>37</v>
-      </c>
       <c r="F46" s="18" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="G46" s="17"/>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="15" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="B47" s="16"/>
       <c r="C47" s="16"/>
@@ -3463,16 +3432,16 @@
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="17"/>
       <c r="B48" s="17" t="s">
+        <v>220</v>
+      </c>
+      <c r="C48" s="17" t="s">
         <v>221</v>
       </c>
-      <c r="C48" s="17" t="s">
+      <c r="D48" s="17" t="s">
+        <v>73</v>
+      </c>
+      <c r="E48" s="17" t="s">
         <v>222</v>
-      </c>
-      <c r="D48" s="17" t="s">
-        <v>75</v>
-      </c>
-      <c r="E48" s="17" t="s">
-        <v>223</v>
       </c>
       <c r="F48" s="17"/>
       <c r="G48" s="17"/>
@@ -3480,16 +3449,16 @@
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="17"/>
       <c r="B49" s="17" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="C49" s="17" t="s">
+        <v>221</v>
+      </c>
+      <c r="D49" s="17" t="s">
+        <v>73</v>
+      </c>
+      <c r="E49" s="17" t="s">
         <v>222</v>
-      </c>
-      <c r="D49" s="17" t="s">
-        <v>75</v>
-      </c>
-      <c r="E49" s="17" t="s">
-        <v>223</v>
       </c>
       <c r="F49" s="17"/>
       <c r="G49" s="17"/>
@@ -3497,16 +3466,16 @@
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="17"/>
       <c r="B50" s="17" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="C50" s="17" t="s">
+        <v>221</v>
+      </c>
+      <c r="D50" s="17" t="s">
+        <v>73</v>
+      </c>
+      <c r="E50" s="17" t="s">
         <v>222</v>
-      </c>
-      <c r="D50" s="17" t="s">
-        <v>75</v>
-      </c>
-      <c r="E50" s="17" t="s">
-        <v>223</v>
       </c>
       <c r="F50" s="17"/>
       <c r="G50" s="17"/>
@@ -3514,16 +3483,16 @@
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="17"/>
       <c r="B51" s="17" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="C51" s="17" t="s">
+        <v>221</v>
+      </c>
+      <c r="D51" s="17" t="s">
+        <v>73</v>
+      </c>
+      <c r="E51" s="17" t="s">
         <v>222</v>
-      </c>
-      <c r="D51" s="17" t="s">
-        <v>75</v>
-      </c>
-      <c r="E51" s="17" t="s">
-        <v>223</v>
       </c>
       <c r="F51" s="17"/>
       <c r="G51" s="17"/>
@@ -3531,16 +3500,16 @@
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="17"/>
       <c r="B52" s="17" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="C52" s="17" t="s">
+        <v>221</v>
+      </c>
+      <c r="D52" s="17" t="s">
+        <v>73</v>
+      </c>
+      <c r="E52" s="17" t="s">
         <v>222</v>
-      </c>
-      <c r="D52" s="17" t="s">
-        <v>75</v>
-      </c>
-      <c r="E52" s="17" t="s">
-        <v>223</v>
       </c>
       <c r="F52" s="17"/>
       <c r="G52" s="17"/>
@@ -3548,16 +3517,16 @@
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="17"/>
       <c r="B53" s="17" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="C53" s="17" t="s">
+        <v>221</v>
+      </c>
+      <c r="D53" s="17" t="s">
+        <v>73</v>
+      </c>
+      <c r="E53" s="17" t="s">
         <v>222</v>
-      </c>
-      <c r="D53" s="17" t="s">
-        <v>75</v>
-      </c>
-      <c r="E53" s="17" t="s">
-        <v>223</v>
       </c>
       <c r="F53" s="17"/>
       <c r="G53" s="17"/>
@@ -3565,16 +3534,16 @@
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="17"/>
       <c r="B54" s="17" t="s">
+        <v>228</v>
+      </c>
+      <c r="C54" s="17" t="s">
         <v>229</v>
       </c>
-      <c r="C54" s="17" t="s">
+      <c r="D54" s="17" t="s">
+        <v>69</v>
+      </c>
+      <c r="E54" s="17" t="s">
         <v>230</v>
-      </c>
-      <c r="D54" s="17" t="s">
-        <v>71</v>
-      </c>
-      <c r="E54" s="17" t="s">
-        <v>231</v>
       </c>
       <c r="F54" s="17"/>
       <c r="G54" s="17"/>
@@ -3582,23 +3551,23 @@
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="17"/>
       <c r="B55" s="17" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="C55" s="17" t="s">
+        <v>229</v>
+      </c>
+      <c r="D55" s="17" t="s">
+        <v>69</v>
+      </c>
+      <c r="E55" s="17" t="s">
         <v>230</v>
-      </c>
-      <c r="D55" s="17" t="s">
-        <v>71</v>
-      </c>
-      <c r="E55" s="17" t="s">
-        <v>231</v>
       </c>
       <c r="F55" s="17"/>
       <c r="G55" s="17"/>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="15" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="B56" s="16"/>
       <c r="C56" s="16"/>
@@ -3610,120 +3579,120 @@
     <row r="57" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="17"/>
       <c r="B57" s="17" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C57" s="17" t="s">
+        <v>233</v>
+      </c>
+      <c r="D57" s="17" t="s">
+        <v>78</v>
+      </c>
+      <c r="E57" s="17" t="s">
         <v>234</v>
       </c>
-      <c r="D57" s="17" t="s">
-        <v>80</v>
-      </c>
-      <c r="E57" s="17" t="s">
+      <c r="F57" s="18" t="s">
         <v>235</v>
-      </c>
-      <c r="F57" s="18" t="s">
-        <v>236</v>
       </c>
       <c r="G57" s="17"/>
     </row>
     <row r="58" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="17"/>
       <c r="B58" s="17" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="C58" s="17" t="s">
+        <v>236</v>
+      </c>
+      <c r="D58" s="17" t="s">
+        <v>98</v>
+      </c>
+      <c r="E58" s="17" t="s">
+        <v>236</v>
+      </c>
+      <c r="F58" s="18" t="s">
         <v>237</v>
-      </c>
-      <c r="D58" s="17" t="s">
-        <v>100</v>
-      </c>
-      <c r="E58" s="17" t="s">
-        <v>237</v>
-      </c>
-      <c r="F58" s="18" t="s">
-        <v>238</v>
       </c>
       <c r="G58" s="17"/>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="17"/>
       <c r="B59" s="17" t="s">
+        <v>238</v>
+      </c>
+      <c r="C59" s="17" t="s">
         <v>239</v>
       </c>
-      <c r="C59" s="17" t="s">
+      <c r="D59" s="17" t="s">
+        <v>82</v>
+      </c>
+      <c r="E59" s="17" t="s">
+        <v>239</v>
+      </c>
+      <c r="F59" s="18" t="s">
         <v>240</v>
-      </c>
-      <c r="D59" s="17" t="s">
-        <v>84</v>
-      </c>
-      <c r="E59" s="17" t="s">
-        <v>240</v>
-      </c>
-      <c r="F59" s="18" t="s">
-        <v>241</v>
       </c>
       <c r="G59" s="17"/>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="17"/>
       <c r="B60" s="17" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="C60" s="17" t="s">
+        <v>239</v>
+      </c>
+      <c r="D60" s="17" t="s">
+        <v>82</v>
+      </c>
+      <c r="E60" s="17" t="s">
+        <v>239</v>
+      </c>
+      <c r="F60" s="18" t="s">
         <v>240</v>
-      </c>
-      <c r="D60" s="17" t="s">
-        <v>84</v>
-      </c>
-      <c r="E60" s="17" t="s">
-        <v>240</v>
-      </c>
-      <c r="F60" s="18" t="s">
-        <v>241</v>
       </c>
       <c r="G60" s="17"/>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="17"/>
       <c r="B61" s="17" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="C61" s="17" t="s">
+        <v>239</v>
+      </c>
+      <c r="D61" s="17" t="s">
+        <v>82</v>
+      </c>
+      <c r="E61" s="17" t="s">
+        <v>239</v>
+      </c>
+      <c r="F61" s="18" t="s">
         <v>240</v>
-      </c>
-      <c r="D61" s="17" t="s">
-        <v>84</v>
-      </c>
-      <c r="E61" s="17" t="s">
-        <v>240</v>
-      </c>
-      <c r="F61" s="18" t="s">
-        <v>241</v>
       </c>
       <c r="G61" s="17"/>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="17"/>
       <c r="B62" s="17" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="C62" s="17" t="s">
+        <v>239</v>
+      </c>
+      <c r="D62" s="17" t="s">
+        <v>82</v>
+      </c>
+      <c r="E62" s="17" t="s">
+        <v>239</v>
+      </c>
+      <c r="F62" s="18" t="s">
         <v>240</v>
-      </c>
-      <c r="D62" s="17" t="s">
-        <v>84</v>
-      </c>
-      <c r="E62" s="17" t="s">
-        <v>240</v>
-      </c>
-      <c r="F62" s="18" t="s">
-        <v>241</v>
       </c>
       <c r="G62" s="17"/>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="15" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="B63" s="16"/>
       <c r="C63" s="16"/>
@@ -3735,16 +3704,16 @@
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="17"/>
       <c r="B64" s="17" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="C64" s="17" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="D64" s="17" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="E64" s="17" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="F64" s="17"/>
       <c r="G64" s="17"/>
@@ -3752,16 +3721,16 @@
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="17"/>
       <c r="B65" s="17" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="C65" s="17" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="D65" s="17" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="E65" s="17" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="F65" s="17"/>
       <c r="G65" s="17"/>
@@ -3769,23 +3738,23 @@
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="17"/>
       <c r="B66" s="17" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="C66" s="17" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="D66" s="17" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="E66" s="17" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="F66" s="17"/>
       <c r="G66" s="17"/>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="15" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="B67" s="16"/>
       <c r="C67" s="16"/>
@@ -3797,82 +3766,82 @@
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="17"/>
       <c r="B68" s="17" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="C68" s="17" t="s">
+        <v>249</v>
+      </c>
+      <c r="D68" s="17" t="s">
+        <v>65</v>
+      </c>
+      <c r="E68" s="17" t="s">
         <v>250</v>
       </c>
-      <c r="D68" s="17" t="s">
-        <v>67</v>
-      </c>
-      <c r="E68" s="17" t="s">
+      <c r="F68" s="18" t="s">
         <v>251</v>
-      </c>
-      <c r="F68" s="18" t="s">
-        <v>252</v>
       </c>
       <c r="G68" s="17"/>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="17"/>
       <c r="B69" s="17" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C69" s="17" t="s">
+        <v>252</v>
+      </c>
+      <c r="D69" s="17" t="s">
+        <v>57</v>
+      </c>
+      <c r="E69" s="17" t="s">
         <v>253</v>
       </c>
-      <c r="D69" s="17" t="s">
-        <v>59</v>
-      </c>
-      <c r="E69" s="17" t="s">
-        <v>254</v>
-      </c>
       <c r="F69" s="18" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="G69" s="17"/>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="17"/>
       <c r="B70" s="17" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="C70" s="17" t="s">
+        <v>254</v>
+      </c>
+      <c r="D70" s="17" t="s">
+        <v>63</v>
+      </c>
+      <c r="E70" s="17" t="s">
         <v>255</v>
       </c>
-      <c r="D70" s="17" t="s">
-        <v>65</v>
-      </c>
-      <c r="E70" s="17" t="s">
-        <v>256</v>
-      </c>
       <c r="F70" s="18" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="G70" s="17"/>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="17"/>
       <c r="B71" s="17" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="C71" s="17" t="s">
+        <v>256</v>
+      </c>
+      <c r="D71" s="17" t="s">
+        <v>60</v>
+      </c>
+      <c r="E71" s="17" t="s">
         <v>257</v>
       </c>
-      <c r="D71" s="17" t="s">
-        <v>62</v>
-      </c>
-      <c r="E71" s="17" t="s">
-        <v>258</v>
-      </c>
       <c r="F71" s="18" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="G71" s="17"/>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="15" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="B72" s="16"/>
       <c r="C72" s="16"/>
@@ -3884,16 +3853,16 @@
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="17"/>
       <c r="B73" s="17" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="C73" s="17" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="D73" s="17" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="E73" s="17" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="F73" s="17"/>
       <c r="G73" s="17"/>
@@ -3901,101 +3870,101 @@
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="17"/>
       <c r="B74" s="17" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C74" s="17" t="s">
+        <v>260</v>
+      </c>
+      <c r="D74" s="17" t="s">
+        <v>86</v>
+      </c>
+      <c r="E74" s="17" t="s">
+        <v>260</v>
+      </c>
+      <c r="F74" s="18" t="s">
         <v>261</v>
-      </c>
-      <c r="D74" s="17" t="s">
-        <v>88</v>
-      </c>
-      <c r="E74" s="17" t="s">
-        <v>261</v>
-      </c>
-      <c r="F74" s="18" t="s">
-        <v>262</v>
       </c>
       <c r="G74" s="17"/>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="17"/>
       <c r="B75" s="17" t="s">
+        <v>262</v>
+      </c>
+      <c r="C75" s="17" t="s">
         <v>263</v>
       </c>
-      <c r="C75" s="17" t="s">
+      <c r="D75" s="17" t="s">
+        <v>90</v>
+      </c>
+      <c r="E75" s="17" t="s">
         <v>264</v>
       </c>
-      <c r="D75" s="17" t="s">
-        <v>92</v>
-      </c>
-      <c r="E75" s="17" t="s">
-        <v>265</v>
-      </c>
       <c r="F75" s="18" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="G75" s="17"/>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="17"/>
       <c r="B76" s="17" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="C76" s="17" t="s">
+        <v>263</v>
+      </c>
+      <c r="D76" s="17" t="s">
+        <v>90</v>
+      </c>
+      <c r="E76" s="17" t="s">
         <v>264</v>
       </c>
-      <c r="D76" s="17" t="s">
-        <v>92</v>
-      </c>
-      <c r="E76" s="17" t="s">
-        <v>265</v>
-      </c>
       <c r="F76" s="18" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="G76" s="17"/>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="17"/>
       <c r="B77" s="17" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="C77" s="17" t="s">
+        <v>263</v>
+      </c>
+      <c r="D77" s="17" t="s">
+        <v>90</v>
+      </c>
+      <c r="E77" s="17" t="s">
         <v>264</v>
       </c>
-      <c r="D77" s="17" t="s">
-        <v>92</v>
-      </c>
-      <c r="E77" s="17" t="s">
-        <v>265</v>
-      </c>
       <c r="F77" s="18" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="G77" s="17"/>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="17"/>
       <c r="B78" s="17" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="C78" s="17" t="s">
+        <v>267</v>
+      </c>
+      <c r="D78" s="17" t="s">
+        <v>94</v>
+      </c>
+      <c r="E78" s="17" t="s">
         <v>268</v>
       </c>
-      <c r="D78" s="17" t="s">
-        <v>96</v>
-      </c>
-      <c r="E78" s="17" t="s">
+      <c r="F78" s="18" t="s">
         <v>269</v>
-      </c>
-      <c r="F78" s="18" t="s">
-        <v>270</v>
       </c>
       <c r="G78" s="17"/>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="15" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="B79" s="16"/>
       <c r="C79" s="16"/>
@@ -4007,73 +3976,73 @@
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="17"/>
       <c r="B80" s="17" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="C80" s="17" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="D80" s="17" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="E80" s="17" t="s">
+        <v>271</v>
+      </c>
+      <c r="F80" s="18" t="s">
         <v>272</v>
-      </c>
-      <c r="F80" s="18" t="s">
-        <v>273</v>
       </c>
       <c r="G80" s="17"/>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="17"/>
       <c r="B81" s="17" t="s">
+        <v>273</v>
+      </c>
+      <c r="C81" s="17" t="s">
+        <v>273</v>
+      </c>
+      <c r="D81" s="17" t="s">
+        <v>143</v>
+      </c>
+      <c r="E81" s="17" t="s">
         <v>274</v>
       </c>
-      <c r="C81" s="17" t="s">
-        <v>274</v>
-      </c>
-      <c r="D81" s="17" t="s">
-        <v>145</v>
-      </c>
-      <c r="E81" s="17" t="s">
-        <v>275</v>
-      </c>
       <c r="F81" s="18" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="G81" s="17"/>
     </row>
     <row r="82" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="17"/>
       <c r="B82" s="17" t="s">
+        <v>275</v>
+      </c>
+      <c r="C82" s="17" t="s">
+        <v>275</v>
+      </c>
+      <c r="D82" s="17" t="s">
+        <v>143</v>
+      </c>
+      <c r="E82" s="17" t="s">
         <v>276</v>
       </c>
-      <c r="C82" s="17" t="s">
-        <v>276</v>
-      </c>
-      <c r="D82" s="17" t="s">
-        <v>145</v>
-      </c>
-      <c r="E82" s="17" t="s">
-        <v>277</v>
-      </c>
       <c r="F82" s="18" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="G82" s="17"/>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="17"/>
       <c r="B83" s="17" t="s">
+        <v>277</v>
+      </c>
+      <c r="C83" s="17" t="s">
+        <v>277</v>
+      </c>
+      <c r="D83" s="17" t="s">
+        <v>115</v>
+      </c>
+      <c r="E83" s="17" t="s">
         <v>278</v>
-      </c>
-      <c r="C83" s="17" t="s">
-        <v>278</v>
-      </c>
-      <c r="D83" s="17" t="s">
-        <v>117</v>
-      </c>
-      <c r="E83" s="17" t="s">
-        <v>279</v>
       </c>
       <c r="F83" s="17"/>
       <c r="G83" s="17"/>
@@ -4081,16 +4050,16 @@
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="17"/>
       <c r="B84" s="17" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="C84" s="17" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="D84" s="17" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="E84" s="17" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="F84" s="17"/>
       <c r="G84" s="17"/>
@@ -4098,23 +4067,23 @@
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="17"/>
       <c r="B85" s="17" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="C85" s="17" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="D85" s="17" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="E85" s="17" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="F85" s="17"/>
       <c r="G85" s="17"/>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="15" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="B86" s="16"/>
       <c r="C86" s="16"/>
@@ -4126,19 +4095,19 @@
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="17"/>
       <c r="B87" s="17" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="C87" s="17" t="s">
+        <v>282</v>
+      </c>
+      <c r="D87" s="17" t="s">
+        <v>147</v>
+      </c>
+      <c r="E87" s="17" t="s">
         <v>283</v>
       </c>
-      <c r="D87" s="17" t="s">
-        <v>149</v>
-      </c>
-      <c r="E87" s="17" t="s">
+      <c r="F87" s="18" t="s">
         <v>284</v>
-      </c>
-      <c r="F87" s="18" t="s">
-        <v>285</v>
       </c>
       <c r="G87" s="17"/>
     </row>

</xml_diff>

<commit_message>
AW4 shield: DigiKey BOM (CSV for BOM Manager + xlsx sheet), C4/C9 100uF 16V
- digikey_bom.csv with manufacturer part numbers for every part, matched by
  DigiKey BOM Manager; DigiKey sheet in bom_objednavka.xlsx scales with board count
- C4 47uF/10V -> 100uF/16V so both 6.3 mm caps are the same part and match
  the footprint; board regenerated, ERC/DRC/parity still clean

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QHDQqfFe1juWLgZ1EWa6E5
</commit_message>
<xml_diff>
--- a/aw4_shield/bom_objednavka.xlsx
+++ b/aw4_shield/bom_objednavka.xlsx
@@ -10,9 +10,10 @@
   <sheets>
     <sheet name="Objednávka" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Osazení" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="DigiKey" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Objednávka!$A$5:$I$43</definedName>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Objednávka!$A$5:$I$42</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -58,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="553" uniqueCount="285">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="708" uniqueCount="390">
   <si>
     <t xml:space="preserve">AW4 shield v0.3 (THT, 100×100 mm) – seznam součástek k objednání</t>
   </si>
@@ -237,603 +238,603 @@
     <t xml:space="preserve">Ø5 mm, rozteč 2,0 mm, 105 °C</t>
   </si>
   <si>
+    <t xml:space="preserve">Panasonic EEU-FR1E100</t>
+  </si>
+  <si>
     <t xml:space="preserve">C3</t>
   </si>
   <si>
-    <t xml:space="preserve">Elektrolyt 100 µF / 10 V (i 16 V)</t>
+    <t xml:space="preserve">Elektrolyt 100 µF / 16 V</t>
   </si>
   <si>
     <t xml:space="preserve">Ø6,3 mm, rozteč 2,5 mm, 105 °C</t>
   </si>
   <si>
+    <t xml:space="preserve">Panasonic EEU-FR1C101</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C4 C9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Elektrolyt 470 µF / 25 V</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ø10 mm, rozteč 5 mm, 105 °C, low-ESR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Panasonic EEU-FR1E471</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Feritová perla</t>
+  </si>
+  <si>
+    <t xml:space="preserve">axiální, ≥ 600 Ω @ 100 MHz, ≥ 1 A (montáž nastojato)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">např. Fair-Rite 2743019447</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L1 L2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kondenzátor 100 nF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">keramický, 50 V, X7R, rozteč 2,54 mm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">např. KEMET C320C104K5R5TA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C2 C5 C6 C7 C8 C10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Polovodiče</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LED zelená 3 mm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">indikace READY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">libovolná 3 mm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Optočlen PC817</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DIP-4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PC817C (Sharp / Everlight / Lite-On)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">U3 U4 U5 U6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P-MOSFET IRF4905</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TO-220 – ochrana proti přepólování</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IRF4905PBF (Infineon)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Q1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P-MOSFET IRF9540N</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TO-220 – spínání solenoidů</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IRF9540NPBF (Infineon)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Q3 Q4 Q5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spínaný stabilizátor 5 V / 1 A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">formát 7805 (SIP-3), vstup 6,5–36 V</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Traco TSR 1-2450</t>
+  </si>
+  <si>
+    <t xml:space="preserve">U1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tranzistor NPN BC337</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TO-92, pinout C-B-E (pad 1 = C)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BC337-40</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Q2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mechanické</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Distanční sloupek M3 + šroub</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pro 4 díry M3 v rozích</t>
+  </si>
+  <si>
+    <t xml:space="preserve">libovolné, např. 10 mm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">H1–H4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Patice pro pojistku TR5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rozteč 5,08 mm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Littelfuse 560 (TR5 patice)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pojistka TR5 5 A, pomalá (T)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TR5, rozteč 5,08 mm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Littelfuse řada 372, 5 A T</t>
+  </si>
+  <si>
+    <t xml:space="preserve">do F1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Relé 12 V SPDT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">kontakty 10 A, cívka 12 V</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Omron G5LE-1 DC12 (pinově kompatibilní: Songle SRD-12VDC-SL-C)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">K1 K2 K3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Konektory</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dutinková lišta 1×15 (patice pro Nano)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rozteč 2,54 mm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">libovolná</t>
+  </si>
+  <si>
+    <t xml:space="preserve">U2 (patice)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kabelová část JST-XH 4 pin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pouzdro + 4 kontakty</t>
+  </si>
+  <si>
+    <t xml:space="preserve">JST XHP-4 + 4× SXH-001T-P0.6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">kabel k displeji</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kolíková lišta 1×2 + jumper</t>
+  </si>
+  <si>
+    <t xml:space="preserve">libovolná + zkratovací propojka 2,54</t>
+  </si>
+  <si>
+    <t xml:space="preserve">JP1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kolíková lišta 1×7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rozteč 2,54 mm (volitelné – rezerva)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">libovolná (odlomit z 1×40)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Konektor JST-XH 4 pin (do DPS)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rozteč 2,5 mm, vertikální</t>
+  </si>
+  <si>
+    <t xml:space="preserve">JST B4B-XH-A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Svorkovnice 2 pól</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rozteč 5,08 mm, do DPS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Phoenix Contact MKDS 1,5/2-5,08 (1715721)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Svorkovnice 6 pól</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Phoenix Contact MKDS 1,5/6-5,08 (1715763)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J2 J3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Moduly</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Arduino Nano (ATmega328P, 5 V)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">zasouvá se do patic (viz níže)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Arduino Nano nebo klon s CH340</t>
+  </si>
+  <si>
+    <t xml:space="preserve">U2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Displej Nextion 2,4″</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UART, 5 V</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nextion NX3224T024 (nebo NX4024T032 3,2″)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mimo desku, přes J5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Celkem kusů k objednání:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Součástek osazených na desce (referencí ve schématu): 74</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Postup osazení – od nejnižších součástek po nejvyšší</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Na desce je na potisku vytištěné, co kam patří (sloupec 'Na potisku'). Označení (R18 …) je v osazovacím výkresu docs/aw4_shield_osazovaci_vykres.pdf a v interaktivním BOM.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Krok</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Označení</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Na potisku</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hodnota ve schématu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pozor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Osazeno ✓</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. rezistory</t>
+  </si>
+  <si>
+    <t xml:space="preserve">100k</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0R</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1k</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10k</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">100R</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">330</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2k2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R21</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R22</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R23</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R24</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2. diody</t>
+  </si>
+  <si>
+    <t xml:space="preserve">12V</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BZX55C12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pozor na polaritu – proužek = katoda (K)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P6KE27</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5V6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BZX55C5V6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4148</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">15V</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BZX55C15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4007</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3. keramické C a ferity</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">100n</t>
+  </si>
+  <si>
+    <t xml:space="preserve">100nF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">600R@100MHz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4. optočleny, tranzistor, LED</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LED</t>
+  </si>
+  <si>
+    <t xml:space="preserve">zelená READY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">polarita! kratší nožička / plochá strana = katoda (čtvercový pad)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BC337</t>
+  </si>
+  <si>
+    <t xml:space="preserve">plochá strana podle potisku; nožičky trochu roztáhnout (rozteč 2,54)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">U3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PC817</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tečka = pin 1 (u čtvercového padu)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">U4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">U5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">U6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5. lišty, patice, JST</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J5 Nextion +5V GND RX TX</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J6 rezerva</t>
+  </si>
+  <si>
+    <t xml:space="preserve">JP1 5V -&gt; Nano (jumper)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6. elektrolyty</t>
+  </si>
+  <si>
+    <t xml:space="preserve">470u</t>
+  </si>
+  <si>
+    <t xml:space="preserve">470uF 25V</t>
+  </si>
+  <si>
+    <t xml:space="preserve">polarita! + na označený pad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10u</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10uF 25V</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">100u</t>
+  </si>
+  <si>
+    <t xml:space="preserve">100uF 16V</t>
+  </si>
+  <si>
     <t xml:space="preserve">C9</t>
   </si>
   <si>
-    <t xml:space="preserve">Elektrolyt 47 µF / 10 V (i 16 V)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Elektrolyt 470 µF / 25 V</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ø10 mm, rozteč 5 mm, 105 °C, low-ESR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">např. Panasonic řada FR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Feritová perla</t>
-  </si>
-  <si>
-    <t xml:space="preserve">axiální, ≥ 600 Ω @ 100 MHz, ≥ 1 A (montáž nastojato)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">např. Fair-Rite 2743019447</t>
-  </si>
-  <si>
-    <t xml:space="preserve">L1 L2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kondenzátor 100 nF</t>
-  </si>
-  <si>
-    <t xml:space="preserve">keramický, 50 V, X7R, rozteč 2,54 mm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">např. KEMET C320C104K5R5TA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C2 C5 C6 C7 C8 C10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Polovodiče</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LED zelená 3 mm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">indikace READY</t>
-  </si>
-  <si>
-    <t xml:space="preserve">libovolná 3 mm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">D10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Optočlen PC817</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DIP-4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PC817C (Sharp / Everlight / Lite-On)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">U3 U4 U5 U6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P-MOSFET IRF4905</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TO-220 – ochrana proti přepólování</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IRF4905PBF (Infineon)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Q1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P-MOSFET IRF9540N</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TO-220 – spínání solenoidů</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IRF9540NPBF (Infineon)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Q3 Q4 Q5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Spínaný stabilizátor 5 V / 1 A</t>
-  </si>
-  <si>
-    <t xml:space="preserve">formát 7805 (SIP-3), vstup 6,5–36 V</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Traco TSR 1-2450</t>
-  </si>
-  <si>
-    <t xml:space="preserve">U1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tranzistor NPN BC337</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TO-92, pinout C-B-E (pad 1 = C)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BC337-40</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Q2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mechanické</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Distanční sloupek M3 + šroub</t>
-  </si>
-  <si>
-    <t xml:space="preserve">pro 4 díry M3 v rozích</t>
-  </si>
-  <si>
-    <t xml:space="preserve">libovolné, např. 10 mm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">H1–H4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Patice pro pojistku TR5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rozteč 5,08 mm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Littelfuse 560 (TR5 patice)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pojistka TR5 5 A, pomalá (T)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TR5, rozteč 5,08 mm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Littelfuse řada 372, 5 A T</t>
-  </si>
-  <si>
-    <t xml:space="preserve">do F1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Relé 12 V SPDT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">kontakty 10 A, cívka 12 V</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Omron G5LE-1 DC12 (pinově kompatibilní: Songle SRD-12VDC-SL-C)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">K1 K2 K3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Konektory</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dutinková lišta 1×15 (patice pro Nano)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rozteč 2,54 mm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">libovolná</t>
-  </si>
-  <si>
-    <t xml:space="preserve">U2 (patice)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kabelová část JST-XH 4 pin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">pouzdro + 4 kontakty</t>
-  </si>
-  <si>
-    <t xml:space="preserve">JST XHP-4 + 4× SXH-001T-P0.6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">kabel k displeji</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kolíková lišta 1×2 + jumper</t>
-  </si>
-  <si>
-    <t xml:space="preserve">libovolná + zkratovací propojka 2,54</t>
-  </si>
-  <si>
-    <t xml:space="preserve">JP1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kolíková lišta 1×7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rozteč 2,54 mm (volitelné – rezerva)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">libovolná (odlomit z 1×40)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">J6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Konektor JST-XH 4 pin (do DPS)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rozteč 2,5 mm, vertikální</t>
-  </si>
-  <si>
-    <t xml:space="preserve">JST B4B-XH-A</t>
-  </si>
-  <si>
-    <t xml:space="preserve">J5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Svorkovnice 2 pól</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rozteč 5,08 mm, do DPS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Phoenix Contact MKDS 1,5/2-5,08 (1715721)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">J1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Svorkovnice 6 pól</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Phoenix Contact MKDS 1,5/6-5,08 (1715763)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">J2 J3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Moduly</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Arduino Nano (ATmega328P, 5 V)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">zasouvá se do patic (viz níže)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Arduino Nano nebo klon s CH340</t>
-  </si>
-  <si>
-    <t xml:space="preserve">U2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Displej Nextion 2,4″</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UART, 5 V</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nextion NX3224T024 (nebo NX4024T032 3,2″)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">mimo desku, přes J5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Celkem kusů k objednání:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Součástek osazených na desce (referencí ve schématu): 74</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Postup osazení – od nejnižších součástek po nejvyšší</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Na desce je na potisku vytištěné, co kam patří (sloupec 'Na potisku'). Označení (R18 …) je v osazovacím výkresu docs/aw4_shield_osazovaci_vykres.pdf a v interaktivním BOM.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Krok</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Označení</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Na potisku</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hodnota ve schématu</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pozor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Osazeno ✓</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. rezistory</t>
-  </si>
-  <si>
-    <t xml:space="preserve">100k</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0R</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1k</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10k</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R9</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">100R</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R13</t>
-  </si>
-  <si>
-    <t xml:space="preserve">330</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R14</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2k2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R16</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R17</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R18</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R19</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R20</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R21</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R22</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R23</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R24</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R25</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2. diody</t>
-  </si>
-  <si>
-    <t xml:space="preserve">12V</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BZX55C12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">pozor na polaritu – proužek = katoda (K)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P6KE27</t>
-  </si>
-  <si>
-    <t xml:space="preserve">D3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5V6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BZX55C5V6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">D4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">D5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">D6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">D7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">D8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4148</t>
-  </si>
-  <si>
-    <t xml:space="preserve">D11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">15V</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BZX55C15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">D12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4007</t>
-  </si>
-  <si>
-    <t xml:space="preserve">D13</t>
-  </si>
-  <si>
-    <t xml:space="preserve">D14</t>
-  </si>
-  <si>
-    <t xml:space="preserve">D15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">D16</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3. keramické C a ferity</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">100n</t>
-  </si>
-  <si>
-    <t xml:space="preserve">100nF</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">L1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FB</t>
-  </si>
-  <si>
-    <t xml:space="preserve">600R@100MHz</t>
-  </si>
-  <si>
-    <t xml:space="preserve">L2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4. optočleny, tranzistor, LED</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LED</t>
-  </si>
-  <si>
-    <t xml:space="preserve">zelená READY</t>
-  </si>
-  <si>
-    <t xml:space="preserve">polarita! kratší nožička / plochá strana = katoda (čtvercový pad)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BC337</t>
-  </si>
-  <si>
-    <t xml:space="preserve">plochá strana podle potisku; nožičky trochu roztáhnout (rozteč 2,54)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">U3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PC817</t>
-  </si>
-  <si>
-    <t xml:space="preserve">tečka = pin 1 (u čtvercového padu)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">U4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">U5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">U6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5. lišty, patice, JST</t>
-  </si>
-  <si>
-    <t xml:space="preserve">J5 Nextion +5V GND RX TX</t>
-  </si>
-  <si>
-    <t xml:space="preserve">J6 rezerva</t>
-  </si>
-  <si>
-    <t xml:space="preserve">JP1 5V -&gt; Nano (jumper)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6. elektrolyty</t>
-  </si>
-  <si>
-    <t xml:space="preserve">470u</t>
-  </si>
-  <si>
-    <t xml:space="preserve">470uF 25V</t>
-  </si>
-  <si>
-    <t xml:space="preserve">polarita! + na označený pad</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10u</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10uF 25V</t>
-  </si>
-  <si>
-    <t xml:space="preserve">47u</t>
-  </si>
-  <si>
-    <t xml:space="preserve">47uF 10V</t>
-  </si>
-  <si>
-    <t xml:space="preserve">100u</t>
-  </si>
-  <si>
-    <t xml:space="preserve">100uF 10V</t>
-  </si>
-  <si>
     <t xml:space="preserve">7. TO-220, stabilizátor, patice pojistky</t>
   </si>
   <si>
@@ -913,6 +914,321 @@
   </si>
   <si>
     <t xml:space="preserve">USB směrem k pravé hraně desky</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DigiKey – seznam pro BOM Manager (digikey.com → BOM Manager → Upload, nebo soubor digikey_bom.csv)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Množství = Ks/deska × počet desek (list Objednávka, C2) + rezerva u drobných dílů (G2). DigiKey páruje podle výrobního čísla (MPN). Dostupnost a ceny nebyly ověřené (z tohoto prostředí není DigiKey dostupný) – řádky označené OVĚŘIT zkontrolujte, u ostatních je to běžný katalogový díl.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Manufacturer Part Number</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Manufacturer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quantity</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Customer Reference</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Popis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Poznámka</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2743019447</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fair-Rite</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Feritová perla – axiální, ≥ 600 Ω @ 100 MHz, ≥ 1 A (montáž nastojato)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C320C104K5R5TA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEMET</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kondenzátor 100 nF – keramický, 50 V, X7R, rozteč 2,54 mm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Littelfuse</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Transil (TVS) 27 V – 600 W, jednosměrný, DO-15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BZX55C12-TAP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vishay</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zenerova dioda 12 V – 0,5 W, DO-35</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BZX55C15-TAP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zenerova dioda 15 V – 0,5 W, DO-35</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BZX55C5V6-TAP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zenerova dioda 5,6 V – 0,5 W, DO-35 – ochrana vstupů</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MFR-25FBF52-100K</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yageo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rezistor 100 kΩ – 0,25 W, 1 %, DIN 0207</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MFR-25FBF52-100R</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rezistor 100 Ω – 0,25 W, 1 %, DIN 0207</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MFR-25FBF52-10K</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rezistor 10 kΩ – 0,25 W, 1 %, DIN 0207</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MFR-25FBF52-1K</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rezistor 1 kΩ – 0,25 W, 1 %, DIN 0207</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MFR-25FBF52-2K2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rezistor 2,2 kΩ – 0,25 W, 1 %, DIN 0207</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MFR-25FBF52-330R</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rezistor 330 Ω – 0,25 W, 1 %, metalizovaný, DIN 0207 (montáž nastojato, rozteč 2,54)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ZOR-25-B-52-0R</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rezistor 0 Ω (propojka) – 0,25 W, DIN 0207 – spojuje PGND a GND (lze nahradit drátkem)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1N4007G</t>
+  </si>
+  <si>
+    <t xml:space="preserve">onsemi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dioda 1N4007 – 1 A / 1000 V, DO-41 – flyback solenoidů</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dioda 1N4148 – DO-35</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A000005</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Arduino</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Arduino Nano (ATmega328P, 5 V) – zasouvá se do patic (viz níže)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">originál; klon s CH340 je levnější, ale DigiKey ho nevede</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IRF4905PBF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Infineon</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P-MOSFET IRF4905 – TO-220 – ochrana proti přepólování</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IRF9540NPBF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P-MOSFET IRF9540N – TO-220 – spínání solenoidů</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B4B-XH-A(LF)(SN)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">JST</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Konektor JST-XH 4 pin (do DPS) – rozteč 2,5 mm, vertikální</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SXH-001T-P0.6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">kabel J5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Krimpovací kontakt JST-XH</t>
+  </si>
+  <si>
+    <t xml:space="preserve">XHP-4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pouzdro JST-XH 4 pin (kabelová část)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WP7104GD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kingbright</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LED zelená 3 mm – indikace READY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LTV-817</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lite-On</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Optočlen PC817 – DIP-4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pinově shodný s PC817</t>
+  </si>
+  <si>
+    <t xml:space="preserve">37215000411</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F1 (pojistka)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pojistka TR5 5 A, pomalá</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OVĚŘIT – řada 372, 5 A T</t>
+  </si>
+  <si>
+    <t xml:space="preserve">56000001009</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Patice pro pojistku TR5 – rozteč 5,08 mm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OVĚŘIT – patice TR5 (řada 560)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">G5LE-1 DC12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Omron</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Relé 12 V SPDT – kontakty 10 A, cívka 12 V</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EEU-FR1C101</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Panasonic</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Elektrolyt 100 µF / 16 V – Ø6,3 mm, rozteč 2,5 mm, 105 °C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EEU-FR1E100</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Elektrolyt 10 µF / 25 V – Ø5 mm, rozteč 2,0 mm, 105 °C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EEU-FR1E471</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Elektrolyt 470 µF / 25 V – Ø10 mm, rozteč 5 mm, 105 °C, low-ESR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1715721</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Phoenix Contact</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Svorkovnice 2 pól – rozteč 5,08 mm, do DPS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MKDS 1,5/2-5,08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1715763</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Svorkovnice 6 pól – rozteč 5,08 mm, do DPS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MKDS 1,5/6-5,08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PPTC151LFBN-RC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sullins</t>
+  </si>
+  <si>
+    <t xml:space="preserve">U2 patice</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dutinková lišta 1×15, 2,54 mm (patice Nana)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PRPC040SAAN-RC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J6, JP1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kolíková lišta 1×40, 2,54 mm (odlomit 1×7 a 1×2)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SPC02SYAN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zkratovací propojka 2,54 mm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TSR 1-2450</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Traco Power</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spínaný stabilizátor 5 V / 1 A – formát 7805 (SIP-3), vstup 6,5–36 V</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BC33740TA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tranzistor NPN BC337 – TO-92, pinout C-B-E (pad 1 = C)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mimo DigiKey: displej Nextion NX3224T024 (např. přímo Itead / Nextion, AliExpress, Laskakit), distanční sloupky M3.</t>
   </si>
 </sst>
 </file>
@@ -923,7 +1239,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="General"/>
   </numFmts>
-  <fonts count="16">
+  <fonts count="18">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1029,6 +1345,20 @@
       <family val="0"/>
       <charset val="1"/>
     </font>
+    <font>
+      <b val="true"/>
+      <sz val="13"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <i val="true"/>
+      <sz val="9"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -1111,7 +1441,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="22">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1186,6 +1516,18 @@
     </xf>
     <xf numFmtId="164" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -1477,7 +1819,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:I46"/>
+  <dimension ref="A1:I45"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
@@ -1922,17 +2264,17 @@
         <v>58</v>
       </c>
       <c r="E19" s="10" t="s">
-        <v>16</v>
+        <v>59</v>
       </c>
       <c r="F19" s="11" t="n">
         <v>1</v>
       </c>
       <c r="G19" s="12" t="n">
-        <f aca="false">F19*$C$2+IF(TRUE(),$G$2,0)</f>
-        <v>3</v>
+        <f aca="false">F19*$C$2</f>
+        <v>1</v>
       </c>
       <c r="H19" s="10" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="I19" s="10"/>
     </row>
@@ -1944,23 +2286,23 @@
         <v>56</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D20" s="7" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="E20" s="7" t="s">
-        <v>16</v>
+        <v>63</v>
       </c>
       <c r="F20" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G20" s="9" t="n">
-        <f aca="false">F20*$C$2+IF(TRUE(),$G$2,0)</f>
-        <v>3</v>
+        <f aca="false">F20*$C$2</f>
+        <v>2</v>
       </c>
       <c r="H20" s="7" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="I20" s="7"/>
     </row>
@@ -1972,27 +2314,27 @@
         <v>56</v>
       </c>
       <c r="C21" s="10" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="D21" s="10" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="E21" s="10" t="s">
-        <v>16</v>
+        <v>67</v>
       </c>
       <c r="F21" s="11" t="n">
         <v>1</v>
       </c>
       <c r="G21" s="12" t="n">
-        <f aca="false">F21*$C$2+IF(TRUE(),$G$2,0)</f>
-        <v>3</v>
+        <f aca="false">F21*$C$2</f>
+        <v>1</v>
       </c>
       <c r="H21" s="10" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="I21" s="10"/>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="7" t="n">
         <v>17</v>
       </c>
@@ -2000,27 +2342,27 @@
         <v>56</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="D22" s="7" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="E22" s="7" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="F22" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G22" s="9" t="n">
         <f aca="false">F22*$C$2+IF(TRUE(),$G$2,0)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H22" s="7" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="I22" s="7"/>
     </row>
-    <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="10" t="n">
         <v>18</v>
       </c>
@@ -2028,23 +2370,23 @@
         <v>56</v>
       </c>
       <c r="C23" s="10" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="D23" s="10" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="E23" s="10" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="F23" s="11" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="G23" s="12" t="n">
         <f aca="false">F23*$C$2+IF(TRUE(),$G$2,0)</f>
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="H23" s="10" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="I23" s="10"/>
     </row>
@@ -2053,26 +2395,26 @@
         <v>19</v>
       </c>
       <c r="B24" s="7" t="s">
-        <v>56</v>
+        <v>77</v>
       </c>
       <c r="C24" s="7" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="D24" s="7" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="E24" s="7" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="F24" s="8" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="G24" s="9" t="n">
-        <f aca="false">F24*$C$2+IF(TRUE(),$G$2,0)</f>
-        <v>8</v>
+        <f aca="false">F24*$C$2</f>
+        <v>1</v>
       </c>
       <c r="H24" s="7" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="I24" s="7"/>
     </row>
@@ -2084,23 +2426,23 @@
         <v>77</v>
       </c>
       <c r="C25" s="10" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="D25" s="10" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="E25" s="10" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="F25" s="11" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G25" s="12" t="n">
         <f aca="false">F25*$C$2</f>
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H25" s="10" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="I25" s="10"/>
     </row>
@@ -2112,23 +2454,23 @@
         <v>77</v>
       </c>
       <c r="C26" s="7" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="D26" s="7" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="E26" s="7" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="F26" s="8" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G26" s="9" t="n">
         <f aca="false">F26*$C$2</f>
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H26" s="7" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="I26" s="7"/>
     </row>
@@ -2140,23 +2482,23 @@
         <v>77</v>
       </c>
       <c r="C27" s="10" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="D27" s="10" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="E27" s="10" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="F27" s="11" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G27" s="12" t="n">
         <f aca="false">F27*$C$2</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H27" s="10" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="I27" s="10"/>
     </row>
@@ -2168,23 +2510,23 @@
         <v>77</v>
       </c>
       <c r="C28" s="7" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="D28" s="7" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="E28" s="7" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="F28" s="8" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G28" s="9" t="n">
         <f aca="false">F28*$C$2</f>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H28" s="7" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="I28" s="7"/>
     </row>
@@ -2196,13 +2538,13 @@
         <v>77</v>
       </c>
       <c r="C29" s="10" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="D29" s="10" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="E29" s="10" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="F29" s="11" t="n">
         <v>1</v>
@@ -2212,7 +2554,7 @@
         <v>1</v>
       </c>
       <c r="H29" s="10" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="I29" s="10"/>
     </row>
@@ -2221,26 +2563,26 @@
         <v>25</v>
       </c>
       <c r="B30" s="7" t="s">
-        <v>77</v>
+        <v>102</v>
       </c>
       <c r="C30" s="7" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="D30" s="7" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="E30" s="7" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="F30" s="8" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G30" s="9" t="n">
         <f aca="false">F30*$C$2</f>
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H30" s="7" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="I30" s="7"/>
     </row>
@@ -2252,23 +2594,23 @@
         <v>102</v>
       </c>
       <c r="C31" s="10" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="D31" s="10" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="E31" s="10" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="F31" s="11" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G31" s="12" t="n">
         <f aca="false">F31*$C$2</f>
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H31" s="10" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="I31" s="10"/>
     </row>
@@ -2280,13 +2622,13 @@
         <v>102</v>
       </c>
       <c r="C32" s="7" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="D32" s="7" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="E32" s="7" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="F32" s="8" t="n">
         <v>1</v>
@@ -2296,11 +2638,11 @@
         <v>1</v>
       </c>
       <c r="H32" s="7" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="I32" s="7"/>
     </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="33" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="10" t="n">
         <v>28</v>
       </c>
@@ -2308,23 +2650,23 @@
         <v>102</v>
       </c>
       <c r="C33" s="10" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="D33" s="10" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="E33" s="10" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="F33" s="11" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G33" s="12" t="n">
         <f aca="false">F33*$C$2</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H33" s="10" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="I33" s="10"/>
     </row>
@@ -2333,30 +2675,30 @@
         <v>29</v>
       </c>
       <c r="B34" s="7" t="s">
-        <v>102</v>
+        <v>119</v>
       </c>
       <c r="C34" s="7" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="D34" s="7" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="E34" s="7" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="F34" s="8" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G34" s="9" t="n">
         <f aca="false">F34*$C$2</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H34" s="7" t="s">
-        <v>118</v>
+        <v>123</v>
       </c>
       <c r="I34" s="7"/>
     </row>
-    <row r="35" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="10" t="n">
         <v>30</v>
       </c>
@@ -2364,23 +2706,23 @@
         <v>119</v>
       </c>
       <c r="C35" s="10" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="D35" s="10" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="E35" s="10" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="F35" s="11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G35" s="12" t="n">
         <f aca="false">F35*$C$2</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H35" s="10" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="I35" s="10"/>
     </row>
@@ -2392,13 +2734,13 @@
         <v>119</v>
       </c>
       <c r="C36" s="7" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="D36" s="7" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="E36" s="7" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="F36" s="8" t="n">
         <v>1</v>
@@ -2408,7 +2750,7 @@
         <v>1</v>
       </c>
       <c r="H36" s="7" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="I36" s="7"/>
     </row>
@@ -2420,13 +2762,13 @@
         <v>119</v>
       </c>
       <c r="C37" s="10" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="D37" s="10" t="s">
-        <v>121</v>
+        <v>132</v>
       </c>
       <c r="E37" s="10" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="F37" s="11" t="n">
         <v>1</v>
@@ -2436,7 +2778,7 @@
         <v>1</v>
       </c>
       <c r="H37" s="10" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="I37" s="10"/>
     </row>
@@ -2448,13 +2790,13 @@
         <v>119</v>
       </c>
       <c r="C38" s="7" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="D38" s="7" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="E38" s="7" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="F38" s="8" t="n">
         <v>1</v>
@@ -2464,7 +2806,7 @@
         <v>1</v>
       </c>
       <c r="H38" s="7" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="I38" s="7"/>
     </row>
@@ -2476,13 +2818,13 @@
         <v>119</v>
       </c>
       <c r="C39" s="10" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="D39" s="10" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="E39" s="10" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="F39" s="11" t="n">
         <v>1</v>
@@ -2492,7 +2834,7 @@
         <v>1</v>
       </c>
       <c r="H39" s="10" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="I39" s="10"/>
     </row>
@@ -2504,23 +2846,23 @@
         <v>119</v>
       </c>
       <c r="C40" s="7" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="D40" s="7" t="s">
         <v>140</v>
       </c>
       <c r="E40" s="7" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="F40" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G40" s="9" t="n">
         <f aca="false">F40*$C$2</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H40" s="7" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="I40" s="7"/>
     </row>
@@ -2529,26 +2871,26 @@
         <v>36</v>
       </c>
       <c r="B41" s="10" t="s">
-        <v>119</v>
+        <v>146</v>
       </c>
       <c r="C41" s="10" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="D41" s="10" t="s">
-        <v>140</v>
+        <v>148</v>
       </c>
       <c r="E41" s="10" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="F41" s="11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G41" s="12" t="n">
         <f aca="false">F41*$C$2</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H41" s="10" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
       <c r="I41" s="10"/>
     </row>
@@ -2560,13 +2902,13 @@
         <v>146</v>
       </c>
       <c r="C42" s="7" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="D42" s="7" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="E42" s="7" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="F42" s="8" t="n">
         <v>1</v>
@@ -2576,54 +2918,26 @@
         <v>1</v>
       </c>
       <c r="H42" s="7" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="I42" s="7"/>
     </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="10" t="n">
-        <v>38</v>
-      </c>
-      <c r="B43" s="10" t="s">
-        <v>146</v>
-      </c>
-      <c r="C43" s="10" t="s">
-        <v>151</v>
-      </c>
-      <c r="D43" s="10" t="s">
-        <v>152</v>
-      </c>
-      <c r="E43" s="10" t="s">
-        <v>153</v>
-      </c>
-      <c r="F43" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="G43" s="12" t="n">
-        <f aca="false">F43*$C$2</f>
-        <v>1</v>
-      </c>
-      <c r="H43" s="10" t="s">
-        <v>154</v>
-      </c>
-      <c r="I43" s="10"/>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E44" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="G44" s="2" t="n">
+        <f aca="false">SUM(G6:G42)</f>
+        <v>113</v>
+      </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E45" s="2" t="s">
-        <v>155</v>
-      </c>
-      <c r="G45" s="2" t="n">
-        <f aca="false">SUM(G6:G43)</f>
-        <v>121</v>
-      </c>
-    </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E46" s="13" t="s">
+      <c r="E45" s="13" t="s">
         <v>156</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A5:I43"/>
+  <autoFilter ref="A5:I42"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -3785,7 +4099,7 @@
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="17"/>
       <c r="B69" s="17" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C69" s="17" t="s">
         <v>252</v>
@@ -3804,16 +4118,16 @@
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="17"/>
       <c r="B70" s="17" t="s">
-        <v>64</v>
+        <v>254</v>
       </c>
       <c r="C70" s="17" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="D70" s="17" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="E70" s="17" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="F70" s="18" t="s">
         <v>251</v>
@@ -3823,16 +4137,16 @@
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="17"/>
       <c r="B71" s="17" t="s">
-        <v>62</v>
+        <v>257</v>
       </c>
       <c r="C71" s="17" t="s">
+        <v>255</v>
+      </c>
+      <c r="D71" s="17" t="s">
+        <v>61</v>
+      </c>
+      <c r="E71" s="17" t="s">
         <v>256</v>
-      </c>
-      <c r="D71" s="17" t="s">
-        <v>60</v>
-      </c>
-      <c r="E71" s="17" t="s">
-        <v>257</v>
       </c>
       <c r="F71" s="18" t="s">
         <v>251</v>
@@ -4120,4 +4434,873 @@
     <oddFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:G42"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="58"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="40"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="19" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="5" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="14" t="s">
+        <v>287</v>
+      </c>
+      <c r="B4" s="14" t="s">
+        <v>288</v>
+      </c>
+      <c r="C4" s="14" t="s">
+        <v>9</v>
+      </c>
+      <c r="D4" s="14" t="s">
+        <v>289</v>
+      </c>
+      <c r="E4" s="14" t="s">
+        <v>290</v>
+      </c>
+      <c r="F4" s="14" t="s">
+        <v>291</v>
+      </c>
+      <c r="G4" s="14" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="17" t="s">
+        <v>293</v>
+      </c>
+      <c r="B5" s="17" t="s">
+        <v>294</v>
+      </c>
+      <c r="C5" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="D5" s="20" t="n">
+        <f aca="false">C5*Objednávka!$C$2+Objednávka!$G$2</f>
+        <v>4</v>
+      </c>
+      <c r="E5" s="17" t="s">
+        <v>72</v>
+      </c>
+      <c r="F5" s="17" t="s">
+        <v>295</v>
+      </c>
+      <c r="G5" s="17"/>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="17" t="s">
+        <v>296</v>
+      </c>
+      <c r="B6" s="17" t="s">
+        <v>297</v>
+      </c>
+      <c r="C6" s="17" t="n">
+        <v>6</v>
+      </c>
+      <c r="D6" s="20" t="n">
+        <f aca="false">C6*Objednávka!$C$2+Objednávka!$G$2</f>
+        <v>8</v>
+      </c>
+      <c r="E6" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="F6" s="17" t="s">
+        <v>298</v>
+      </c>
+      <c r="G6" s="17"/>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="17" t="s">
+        <v>43</v>
+      </c>
+      <c r="B7" s="17" t="s">
+        <v>299</v>
+      </c>
+      <c r="C7" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" s="20" t="n">
+        <f aca="false">C7*Objednávka!$C$2+Objednávka!$G$2</f>
+        <v>3</v>
+      </c>
+      <c r="E7" s="17" t="s">
+        <v>44</v>
+      </c>
+      <c r="F7" s="17" t="s">
+        <v>300</v>
+      </c>
+      <c r="G7" s="17"/>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="17" t="s">
+        <v>301</v>
+      </c>
+      <c r="B8" s="17" t="s">
+        <v>302</v>
+      </c>
+      <c r="C8" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" s="20" t="n">
+        <f aca="false">C8*Objednávka!$C$2+Objednávka!$G$2</f>
+        <v>3</v>
+      </c>
+      <c r="E8" s="17" t="s">
+        <v>48</v>
+      </c>
+      <c r="F8" s="17" t="s">
+        <v>303</v>
+      </c>
+      <c r="G8" s="17"/>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="17" t="s">
+        <v>304</v>
+      </c>
+      <c r="B9" s="17" t="s">
+        <v>302</v>
+      </c>
+      <c r="C9" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="D9" s="20" t="n">
+        <f aca="false">C9*Objednávka!$C$2+Objednávka!$G$2</f>
+        <v>5</v>
+      </c>
+      <c r="E9" s="17" t="s">
+        <v>51</v>
+      </c>
+      <c r="F9" s="17" t="s">
+        <v>305</v>
+      </c>
+      <c r="G9" s="17"/>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="17" t="s">
+        <v>306</v>
+      </c>
+      <c r="B10" s="17" t="s">
+        <v>302</v>
+      </c>
+      <c r="C10" s="17" t="n">
+        <v>6</v>
+      </c>
+      <c r="D10" s="20" t="n">
+        <f aca="false">C10*Objednávka!$C$2+Objednávka!$G$2</f>
+        <v>8</v>
+      </c>
+      <c r="E10" s="17" t="s">
+        <v>55</v>
+      </c>
+      <c r="F10" s="17" t="s">
+        <v>307</v>
+      </c>
+      <c r="G10" s="17"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="17" t="s">
+        <v>308</v>
+      </c>
+      <c r="B11" s="17" t="s">
+        <v>309</v>
+      </c>
+      <c r="C11" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" s="20" t="n">
+        <f aca="false">C11*Objednávka!$C$2+Objednávka!$G$2</f>
+        <v>3</v>
+      </c>
+      <c r="E11" s="17" t="s">
+        <v>31</v>
+      </c>
+      <c r="F11" s="17" t="s">
+        <v>310</v>
+      </c>
+      <c r="G11" s="17"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="17" t="s">
+        <v>311</v>
+      </c>
+      <c r="B12" s="17" t="s">
+        <v>309</v>
+      </c>
+      <c r="C12" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="D12" s="20" t="n">
+        <f aca="false">C12*Objednávka!$C$2+Objednávka!$G$2</f>
+        <v>4</v>
+      </c>
+      <c r="E12" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="F12" s="17" t="s">
+        <v>312</v>
+      </c>
+      <c r="G12" s="17"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="17" t="s">
+        <v>313</v>
+      </c>
+      <c r="B13" s="17" t="s">
+        <v>309</v>
+      </c>
+      <c r="C13" s="17" t="n">
+        <v>8</v>
+      </c>
+      <c r="D13" s="20" t="n">
+        <f aca="false">C13*Objednávka!$C$2+Objednávka!$G$2</f>
+        <v>10</v>
+      </c>
+      <c r="E13" s="17" t="s">
+        <v>29</v>
+      </c>
+      <c r="F13" s="17" t="s">
+        <v>314</v>
+      </c>
+      <c r="G13" s="17"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="17" t="s">
+        <v>315</v>
+      </c>
+      <c r="B14" s="17" t="s">
+        <v>309</v>
+      </c>
+      <c r="C14" s="17" t="n">
+        <v>7</v>
+      </c>
+      <c r="D14" s="20" t="n">
+        <f aca="false">C14*Objednávka!$C$2+Objednávka!$G$2</f>
+        <v>9</v>
+      </c>
+      <c r="E14" s="17" t="s">
+        <v>25</v>
+      </c>
+      <c r="F14" s="17" t="s">
+        <v>316</v>
+      </c>
+      <c r="G14" s="17"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="17" t="s">
+        <v>317</v>
+      </c>
+      <c r="B15" s="17" t="s">
+        <v>309</v>
+      </c>
+      <c r="C15" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="D15" s="20" t="n">
+        <f aca="false">C15*Objednávka!$C$2+Objednávka!$G$2</f>
+        <v>4</v>
+      </c>
+      <c r="E15" s="17" t="s">
+        <v>27</v>
+      </c>
+      <c r="F15" s="17" t="s">
+        <v>318</v>
+      </c>
+      <c r="G15" s="17"/>
+    </row>
+    <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="17" t="s">
+        <v>319</v>
+      </c>
+      <c r="B16" s="17" t="s">
+        <v>309</v>
+      </c>
+      <c r="C16" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="D16" s="20" t="n">
+        <f aca="false">C16*Objednávka!$C$2+Objednávka!$G$2</f>
+        <v>6</v>
+      </c>
+      <c r="E16" s="17" t="s">
+        <v>23</v>
+      </c>
+      <c r="F16" s="17" t="s">
+        <v>320</v>
+      </c>
+      <c r="G16" s="17"/>
+    </row>
+    <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="17" t="s">
+        <v>321</v>
+      </c>
+      <c r="B17" s="17" t="s">
+        <v>309</v>
+      </c>
+      <c r="C17" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="D17" s="20" t="n">
+        <f aca="false">C17*Objednávka!$C$2+Objednávka!$G$2</f>
+        <v>3</v>
+      </c>
+      <c r="E17" s="17" t="s">
+        <v>17</v>
+      </c>
+      <c r="F17" s="17" t="s">
+        <v>322</v>
+      </c>
+      <c r="G17" s="17"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="17" t="s">
+        <v>323</v>
+      </c>
+      <c r="B18" s="17" t="s">
+        <v>324</v>
+      </c>
+      <c r="C18" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="D18" s="20" t="n">
+        <f aca="false">C18*Objednávka!$C$2+Objednávka!$G$2</f>
+        <v>5</v>
+      </c>
+      <c r="E18" s="17" t="s">
+        <v>36</v>
+      </c>
+      <c r="F18" s="17" t="s">
+        <v>325</v>
+      </c>
+      <c r="G18" s="17"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="17" t="s">
+        <v>39</v>
+      </c>
+      <c r="B19" s="17" t="s">
+        <v>324</v>
+      </c>
+      <c r="C19" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="D19" s="20" t="n">
+        <f aca="false">C19*Objednávka!$C$2+Objednávka!$G$2</f>
+        <v>3</v>
+      </c>
+      <c r="E19" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="F19" s="17" t="s">
+        <v>326</v>
+      </c>
+      <c r="G19" s="17"/>
+    </row>
+    <row r="20" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="17" t="s">
+        <v>327</v>
+      </c>
+      <c r="B20" s="17" t="s">
+        <v>328</v>
+      </c>
+      <c r="C20" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="D20" s="20" t="n">
+        <f aca="false">C20*Objednávka!$C$2</f>
+        <v>1</v>
+      </c>
+      <c r="E20" s="17" t="s">
+        <v>150</v>
+      </c>
+      <c r="F20" s="17" t="s">
+        <v>329</v>
+      </c>
+      <c r="G20" s="17" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="17" t="s">
+        <v>331</v>
+      </c>
+      <c r="B21" s="17" t="s">
+        <v>332</v>
+      </c>
+      <c r="C21" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="D21" s="20" t="n">
+        <f aca="false">C21*Objednávka!$C$2</f>
+        <v>1</v>
+      </c>
+      <c r="E21" s="17" t="s">
+        <v>89</v>
+      </c>
+      <c r="F21" s="17" t="s">
+        <v>333</v>
+      </c>
+      <c r="G21" s="17"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="17" t="s">
+        <v>334</v>
+      </c>
+      <c r="B22" s="17" t="s">
+        <v>332</v>
+      </c>
+      <c r="C22" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="D22" s="20" t="n">
+        <f aca="false">C22*Objednávka!$C$2</f>
+        <v>3</v>
+      </c>
+      <c r="E22" s="17" t="s">
+        <v>93</v>
+      </c>
+      <c r="F22" s="17" t="s">
+        <v>335</v>
+      </c>
+      <c r="G22" s="17"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="17" t="s">
+        <v>336</v>
+      </c>
+      <c r="B23" s="17" t="s">
+        <v>337</v>
+      </c>
+      <c r="C23" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="D23" s="20" t="n">
+        <f aca="false">C23*Objednávka!$C$2</f>
+        <v>1</v>
+      </c>
+      <c r="E23" s="17" t="s">
+        <v>138</v>
+      </c>
+      <c r="F23" s="17" t="s">
+        <v>338</v>
+      </c>
+      <c r="G23" s="17"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="17" t="s">
+        <v>339</v>
+      </c>
+      <c r="B24" s="17" t="s">
+        <v>337</v>
+      </c>
+      <c r="C24" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="D24" s="20" t="n">
+        <f aca="false">C24*Objednávka!$C$2</f>
+        <v>4</v>
+      </c>
+      <c r="E24" s="17" t="s">
+        <v>340</v>
+      </c>
+      <c r="F24" s="17" t="s">
+        <v>341</v>
+      </c>
+      <c r="G24" s="17"/>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="17" t="s">
+        <v>342</v>
+      </c>
+      <c r="B25" s="17" t="s">
+        <v>337</v>
+      </c>
+      <c r="C25" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="D25" s="20" t="n">
+        <f aca="false">C25*Objednávka!$C$2</f>
+        <v>1</v>
+      </c>
+      <c r="E25" s="17" t="s">
+        <v>340</v>
+      </c>
+      <c r="F25" s="17" t="s">
+        <v>343</v>
+      </c>
+      <c r="G25" s="17"/>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="17" t="s">
+        <v>344</v>
+      </c>
+      <c r="B26" s="17" t="s">
+        <v>345</v>
+      </c>
+      <c r="C26" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="D26" s="20" t="n">
+        <f aca="false">C26*Objednávka!$C$2</f>
+        <v>1</v>
+      </c>
+      <c r="E26" s="17" t="s">
+        <v>81</v>
+      </c>
+      <c r="F26" s="17" t="s">
+        <v>346</v>
+      </c>
+      <c r="G26" s="17"/>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="17" t="s">
+        <v>347</v>
+      </c>
+      <c r="B27" s="17" t="s">
+        <v>348</v>
+      </c>
+      <c r="C27" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="D27" s="20" t="n">
+        <f aca="false">C27*Objednávka!$C$2</f>
+        <v>4</v>
+      </c>
+      <c r="E27" s="17" t="s">
+        <v>85</v>
+      </c>
+      <c r="F27" s="17" t="s">
+        <v>349</v>
+      </c>
+      <c r="G27" s="17" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="17" t="s">
+        <v>351</v>
+      </c>
+      <c r="B28" s="17" t="s">
+        <v>299</v>
+      </c>
+      <c r="C28" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="D28" s="20" t="n">
+        <f aca="false">C28*Objednávka!$C$2</f>
+        <v>1</v>
+      </c>
+      <c r="E28" s="17" t="s">
+        <v>352</v>
+      </c>
+      <c r="F28" s="17" t="s">
+        <v>353</v>
+      </c>
+      <c r="G28" s="18" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="17" t="s">
+        <v>355</v>
+      </c>
+      <c r="B29" s="17" t="s">
+        <v>299</v>
+      </c>
+      <c r="C29" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="D29" s="20" t="n">
+        <f aca="false">C29*Objednávka!$C$2</f>
+        <v>1</v>
+      </c>
+      <c r="E29" s="17" t="s">
+        <v>110</v>
+      </c>
+      <c r="F29" s="17" t="s">
+        <v>356</v>
+      </c>
+      <c r="G29" s="18" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="17" t="s">
+        <v>358</v>
+      </c>
+      <c r="B30" s="17" t="s">
+        <v>359</v>
+      </c>
+      <c r="C30" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="D30" s="20" t="n">
+        <f aca="false">C30*Objednávka!$C$2</f>
+        <v>3</v>
+      </c>
+      <c r="E30" s="17" t="s">
+        <v>118</v>
+      </c>
+      <c r="F30" s="17" t="s">
+        <v>360</v>
+      </c>
+      <c r="G30" s="17"/>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="17" t="s">
+        <v>361</v>
+      </c>
+      <c r="B31" s="17" t="s">
+        <v>362</v>
+      </c>
+      <c r="C31" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="D31" s="20" t="n">
+        <f aca="false">C31*Objednávka!$C$2</f>
+        <v>2</v>
+      </c>
+      <c r="E31" s="17" t="s">
+        <v>64</v>
+      </c>
+      <c r="F31" s="17" t="s">
+        <v>363</v>
+      </c>
+      <c r="G31" s="17"/>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="17" t="s">
+        <v>364</v>
+      </c>
+      <c r="B32" s="17" t="s">
+        <v>362</v>
+      </c>
+      <c r="C32" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="D32" s="20" t="n">
+        <f aca="false">C32*Objednávka!$C$2</f>
+        <v>1</v>
+      </c>
+      <c r="E32" s="17" t="s">
+        <v>60</v>
+      </c>
+      <c r="F32" s="17" t="s">
+        <v>365</v>
+      </c>
+      <c r="G32" s="17"/>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="17" t="s">
+        <v>366</v>
+      </c>
+      <c r="B33" s="17" t="s">
+        <v>362</v>
+      </c>
+      <c r="C33" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="D33" s="20" t="n">
+        <f aca="false">C33*Objednávka!$C$2</f>
+        <v>1</v>
+      </c>
+      <c r="E33" s="17" t="s">
+        <v>68</v>
+      </c>
+      <c r="F33" s="17" t="s">
+        <v>367</v>
+      </c>
+      <c r="G33" s="17"/>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="17" t="s">
+        <v>368</v>
+      </c>
+      <c r="B34" s="17" t="s">
+        <v>369</v>
+      </c>
+      <c r="C34" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="D34" s="20" t="n">
+        <f aca="false">C34*Objednávka!$C$2</f>
+        <v>1</v>
+      </c>
+      <c r="E34" s="17" t="s">
+        <v>142</v>
+      </c>
+      <c r="F34" s="17" t="s">
+        <v>370</v>
+      </c>
+      <c r="G34" s="17" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="17" t="s">
+        <v>372</v>
+      </c>
+      <c r="B35" s="17" t="s">
+        <v>369</v>
+      </c>
+      <c r="C35" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="D35" s="20" t="n">
+        <f aca="false">C35*Objednávka!$C$2</f>
+        <v>2</v>
+      </c>
+      <c r="E35" s="17" t="s">
+        <v>145</v>
+      </c>
+      <c r="F35" s="17" t="s">
+        <v>373</v>
+      </c>
+      <c r="G35" s="17" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="17" t="s">
+        <v>375</v>
+      </c>
+      <c r="B36" s="17" t="s">
+        <v>376</v>
+      </c>
+      <c r="C36" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="D36" s="20" t="n">
+        <f aca="false">C36*Objednávka!$C$2</f>
+        <v>2</v>
+      </c>
+      <c r="E36" s="17" t="s">
+        <v>377</v>
+      </c>
+      <c r="F36" s="17" t="s">
+        <v>378</v>
+      </c>
+      <c r="G36" s="17"/>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="17" t="s">
+        <v>379</v>
+      </c>
+      <c r="B37" s="17" t="s">
+        <v>376</v>
+      </c>
+      <c r="C37" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="D37" s="20" t="n">
+        <f aca="false">C37*Objednávka!$C$2</f>
+        <v>1</v>
+      </c>
+      <c r="E37" s="17" t="s">
+        <v>380</v>
+      </c>
+      <c r="F37" s="17" t="s">
+        <v>381</v>
+      </c>
+      <c r="G37" s="17"/>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="17" t="s">
+        <v>382</v>
+      </c>
+      <c r="B38" s="17" t="s">
+        <v>376</v>
+      </c>
+      <c r="C38" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="D38" s="20" t="n">
+        <f aca="false">C38*Objednávka!$C$2</f>
+        <v>1</v>
+      </c>
+      <c r="E38" s="17" t="s">
+        <v>130</v>
+      </c>
+      <c r="F38" s="17" t="s">
+        <v>383</v>
+      </c>
+      <c r="G38" s="17"/>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="17" t="s">
+        <v>384</v>
+      </c>
+      <c r="B39" s="17" t="s">
+        <v>385</v>
+      </c>
+      <c r="C39" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="D39" s="20" t="n">
+        <f aca="false">C39*Objednávka!$C$2</f>
+        <v>1</v>
+      </c>
+      <c r="E39" s="17" t="s">
+        <v>97</v>
+      </c>
+      <c r="F39" s="17" t="s">
+        <v>386</v>
+      </c>
+      <c r="G39" s="17"/>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="17" t="s">
+        <v>387</v>
+      </c>
+      <c r="B40" s="17" t="s">
+        <v>324</v>
+      </c>
+      <c r="C40" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="D40" s="20" t="n">
+        <f aca="false">C40*Objednávka!$C$2</f>
+        <v>1</v>
+      </c>
+      <c r="E40" s="17" t="s">
+        <v>101</v>
+      </c>
+      <c r="F40" s="17" t="s">
+        <v>388</v>
+      </c>
+      <c r="G40" s="17"/>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="21" t="s">
+        <v>389</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
AW4 shield: DigiKey BOM - C3 10uF/25V is Panasonic ECA-1EM100, add alternatives column
EEU-FR1E100 is not a valid part number. Added a column with drop-in
alternatives (same value, package and lead pitch) for the electrolytics and
the parts whose numbers could not be checked.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QHDQqfFe1juWLgZ1EWa6E5
</commit_message>
<xml_diff>
--- a/aw4_shield/bom_objednavka.xlsx
+++ b/aw4_shield/bom_objednavka.xlsx
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="708" uniqueCount="390">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="718" uniqueCount="400">
   <si>
     <t xml:space="preserve">AW4 shield v0.3 (THT, 100×100 mm) – seznam součástek k objednání</t>
   </si>
@@ -235,10 +235,10 @@
     <t xml:space="preserve">Elektrolyt 10 µF / 25 V</t>
   </si>
   <si>
-    <t xml:space="preserve">Ø5 mm, rozteč 2,0 mm, 105 °C</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Panasonic EEU-FR1E100</t>
+    <t xml:space="preserve">Ø5 mm, rozteč 2,0 mm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Panasonic ECA-1EM100</t>
   </si>
   <si>
     <t xml:space="preserve">C3</t>
@@ -940,6 +940,9 @@
     <t xml:space="preserve">Poznámka</t>
   </si>
   <si>
+    <t xml:space="preserve">Náhrada, když DigiKey díl nezná / nemá</t>
+  </si>
+  <si>
     <t xml:space="preserve">2743019447</t>
   </si>
   <si>
@@ -949,6 +952,9 @@
     <t xml:space="preserve">Feritová perla – axiální, ≥ 600 Ω @ 100 MHz, ≥ 1 A (montáž nastojato)</t>
   </si>
   <si>
+    <t xml:space="preserve">Würth 74270012 (feritová perla)</t>
+  </si>
+  <si>
     <t xml:space="preserve">C320C104K5R5TA</t>
   </si>
   <si>
@@ -1102,6 +1108,9 @@
     <t xml:space="preserve">LED zelená 3 mm – indikace READY</t>
   </si>
   <si>
+    <t xml:space="preserve">libovolná zelená LED 3 mm</t>
+  </si>
+  <si>
     <t xml:space="preserve">LTV-817</t>
   </si>
   <si>
@@ -1114,6 +1123,9 @@
     <t xml:space="preserve">pinově shodný s PC817</t>
   </si>
   <si>
+    <t xml:space="preserve">Sharp PC817X1NSZ1B</t>
+  </si>
+  <si>
     <t xml:space="preserve">37215000411</t>
   </si>
   <si>
@@ -1126,6 +1138,9 @@
     <t xml:space="preserve">OVĚŘIT – řada 372, 5 A T</t>
   </si>
   <si>
+    <t xml:space="preserve">libovolná pojistka TR5 5 A T</t>
+  </si>
+  <si>
     <t xml:space="preserve">56000001009</t>
   </si>
   <si>
@@ -1135,6 +1150,9 @@
     <t xml:space="preserve">OVĚŘIT – patice TR5 (řada 560)</t>
   </si>
   <si>
+    <t xml:space="preserve">libovolná patice TR5, rozteč 5,08 mm</t>
+  </si>
+  <si>
     <t xml:space="preserve">G5LE-1 DC12</t>
   </si>
   <si>
@@ -1144,25 +1162,37 @@
     <t xml:space="preserve">Relé 12 V SPDT – kontakty 10 A, cívka 12 V</t>
   </si>
   <si>
+    <t xml:space="preserve">ECA-1EM100</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Panasonic</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Elektrolyt 10 µF / 25 V – Ø5 mm, rozteč 2,0 mm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ø5×11 mm, rozteč 2,0 mm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nichicon UVR1E100MDD</t>
+  </si>
+  <si>
     <t xml:space="preserve">EEU-FR1C101</t>
   </si>
   <si>
-    <t xml:space="preserve">Panasonic</t>
-  </si>
-  <si>
     <t xml:space="preserve">Elektrolyt 100 µF / 16 V – Ø6,3 mm, rozteč 2,5 mm, 105 °C</t>
   </si>
   <si>
-    <t xml:space="preserve">EEU-FR1E100</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Elektrolyt 10 µF / 25 V – Ø5 mm, rozteč 2,0 mm, 105 °C</t>
+    <t xml:space="preserve">Nichicon UVR1C101MED</t>
   </si>
   <si>
     <t xml:space="preserve">EEU-FR1E471</t>
   </si>
   <si>
     <t xml:space="preserve">Elektrolyt 470 µF / 25 V – Ø10 mm, rozteč 5 mm, 105 °C, low-ESR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nichicon UHE1E471MPD</t>
   </si>
   <si>
     <t xml:space="preserve">1715721</t>
@@ -4441,7 +4471,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G42"/>
+  <dimension ref="A1:H42"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="24"/>
@@ -4449,7 +4479,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="9"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="30"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="58"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="0" width="34"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4484,13 +4514,16 @@
       <c r="G4" s="14" t="s">
         <v>292</v>
       </c>
+      <c r="H4" s="14" t="s">
+        <v>293</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="17" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="B5" s="17" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="C5" s="17" t="n">
         <v>2</v>
@@ -4503,16 +4536,19 @@
         <v>72</v>
       </c>
       <c r="F5" s="17" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="G5" s="17"/>
+      <c r="H5" s="17" t="s">
+        <v>297</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="17" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="B6" s="17" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="C6" s="17" t="n">
         <v>6</v>
@@ -4525,16 +4561,17 @@
         <v>76</v>
       </c>
       <c r="F6" s="17" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="G6" s="17"/>
+      <c r="H6" s="17"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="17" t="s">
         <v>43</v>
       </c>
       <c r="B7" s="17" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="C7" s="17" t="n">
         <v>1</v>
@@ -4547,16 +4584,17 @@
         <v>44</v>
       </c>
       <c r="F7" s="17" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="G7" s="17"/>
+      <c r="H7" s="17"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="17" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="B8" s="17" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="C8" s="17" t="n">
         <v>1</v>
@@ -4569,16 +4607,17 @@
         <v>48</v>
       </c>
       <c r="F8" s="17" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="G8" s="17"/>
+      <c r="H8" s="17"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="17" t="s">
+        <v>306</v>
+      </c>
+      <c r="B9" s="17" t="s">
         <v>304</v>
-      </c>
-      <c r="B9" s="17" t="s">
-        <v>302</v>
       </c>
       <c r="C9" s="17" t="n">
         <v>3</v>
@@ -4591,16 +4630,17 @@
         <v>51</v>
       </c>
       <c r="F9" s="17" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="G9" s="17"/>
+      <c r="H9" s="17"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="17" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="B10" s="17" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="C10" s="17" t="n">
         <v>6</v>
@@ -4613,16 +4653,17 @@
         <v>55</v>
       </c>
       <c r="F10" s="17" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="G10" s="17"/>
+      <c r="H10" s="17"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="17" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="B11" s="17" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="C11" s="17" t="n">
         <v>1</v>
@@ -4635,16 +4676,17 @@
         <v>31</v>
       </c>
       <c r="F11" s="17" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="G11" s="17"/>
+      <c r="H11" s="17"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="17" t="s">
+        <v>313</v>
+      </c>
+      <c r="B12" s="17" t="s">
         <v>311</v>
-      </c>
-      <c r="B12" s="17" t="s">
-        <v>309</v>
       </c>
       <c r="C12" s="17" t="n">
         <v>2</v>
@@ -4657,16 +4699,17 @@
         <v>20</v>
       </c>
       <c r="F12" s="17" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="G12" s="17"/>
+      <c r="H12" s="17"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="17" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="B13" s="17" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="C13" s="17" t="n">
         <v>8</v>
@@ -4679,16 +4722,17 @@
         <v>29</v>
       </c>
       <c r="F13" s="17" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="G13" s="17"/>
+      <c r="H13" s="17"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="17" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="B14" s="17" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="C14" s="17" t="n">
         <v>7</v>
@@ -4701,16 +4745,17 @@
         <v>25</v>
       </c>
       <c r="F14" s="17" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="G14" s="17"/>
+      <c r="H14" s="17"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="17" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="B15" s="17" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="C15" s="17" t="n">
         <v>2</v>
@@ -4723,16 +4768,17 @@
         <v>27</v>
       </c>
       <c r="F15" s="17" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="G15" s="17"/>
+      <c r="H15" s="17"/>
     </row>
     <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="17" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="B16" s="17" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="C16" s="17" t="n">
         <v>4</v>
@@ -4745,16 +4791,17 @@
         <v>23</v>
       </c>
       <c r="F16" s="17" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="G16" s="17"/>
+      <c r="H16" s="17"/>
     </row>
     <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="17" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="B17" s="17" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="C17" s="17" t="n">
         <v>1</v>
@@ -4767,16 +4814,17 @@
         <v>17</v>
       </c>
       <c r="F17" s="17" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="G17" s="17"/>
+      <c r="H17" s="17"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="17" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="B18" s="17" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="C18" s="17" t="n">
         <v>3</v>
@@ -4789,16 +4837,17 @@
         <v>36</v>
       </c>
       <c r="F18" s="17" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="G18" s="17"/>
+      <c r="H18" s="17"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="17" t="s">
         <v>39</v>
       </c>
       <c r="B19" s="17" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="C19" s="17" t="n">
         <v>1</v>
@@ -4811,16 +4860,17 @@
         <v>40</v>
       </c>
       <c r="F19" s="17" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="G19" s="17"/>
+      <c r="H19" s="17"/>
     </row>
     <row r="20" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="17" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="B20" s="17" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="C20" s="17" t="n">
         <v>1</v>
@@ -4833,18 +4883,19 @@
         <v>150</v>
       </c>
       <c r="F20" s="17" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="G20" s="17" t="s">
-        <v>330</v>
-      </c>
+        <v>332</v>
+      </c>
+      <c r="H20" s="17"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="17" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="B21" s="17" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="C21" s="17" t="n">
         <v>1</v>
@@ -4857,16 +4908,17 @@
         <v>89</v>
       </c>
       <c r="F21" s="17" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="G21" s="17"/>
+      <c r="H21" s="17"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="17" t="s">
+        <v>336</v>
+      </c>
+      <c r="B22" s="17" t="s">
         <v>334</v>
-      </c>
-      <c r="B22" s="17" t="s">
-        <v>332</v>
       </c>
       <c r="C22" s="17" t="n">
         <v>3</v>
@@ -4879,16 +4931,17 @@
         <v>93</v>
       </c>
       <c r="F22" s="17" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="G22" s="17"/>
+      <c r="H22" s="17"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="17" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="B23" s="17" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="C23" s="17" t="n">
         <v>1</v>
@@ -4901,16 +4954,17 @@
         <v>138</v>
       </c>
       <c r="F23" s="17" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="G23" s="17"/>
+      <c r="H23" s="17"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="17" t="s">
+        <v>341</v>
+      </c>
+      <c r="B24" s="17" t="s">
         <v>339</v>
-      </c>
-      <c r="B24" s="17" t="s">
-        <v>337</v>
       </c>
       <c r="C24" s="17" t="n">
         <v>4</v>
@@ -4920,19 +4974,20 @@
         <v>4</v>
       </c>
       <c r="E24" s="17" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="F24" s="17" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="G24" s="17"/>
+      <c r="H24" s="17"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="17" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="B25" s="17" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="C25" s="17" t="n">
         <v>1</v>
@@ -4942,19 +4997,20 @@
         <v>1</v>
       </c>
       <c r="E25" s="17" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="F25" s="17" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="G25" s="17"/>
+      <c r="H25" s="17"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="17" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="B26" s="17" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="C26" s="17" t="n">
         <v>1</v>
@@ -4967,16 +5023,19 @@
         <v>81</v>
       </c>
       <c r="F26" s="17" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="G26" s="17"/>
+      <c r="H26" s="17" t="s">
+        <v>349</v>
+      </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="17" t="s">
-        <v>347</v>
+        <v>350</v>
       </c>
       <c r="B27" s="17" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="C27" s="17" t="n">
         <v>4</v>
@@ -4989,18 +5048,21 @@
         <v>85</v>
       </c>
       <c r="F27" s="17" t="s">
-        <v>349</v>
+        <v>352</v>
       </c>
       <c r="G27" s="17" t="s">
-        <v>350</v>
+        <v>353</v>
+      </c>
+      <c r="H27" s="17" t="s">
+        <v>354</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="17" t="s">
-        <v>351</v>
+        <v>355</v>
       </c>
       <c r="B28" s="17" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="C28" s="17" t="n">
         <v>1</v>
@@ -5010,21 +5072,24 @@
         <v>1</v>
       </c>
       <c r="E28" s="17" t="s">
-        <v>352</v>
+        <v>356</v>
       </c>
       <c r="F28" s="17" t="s">
-        <v>353</v>
+        <v>357</v>
       </c>
       <c r="G28" s="18" t="s">
-        <v>354</v>
+        <v>358</v>
+      </c>
+      <c r="H28" s="17" t="s">
+        <v>359</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="17" t="s">
-        <v>355</v>
+        <v>360</v>
       </c>
       <c r="B29" s="17" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="C29" s="17" t="n">
         <v>1</v>
@@ -5037,18 +5102,21 @@
         <v>110</v>
       </c>
       <c r="F29" s="17" t="s">
-        <v>356</v>
+        <v>361</v>
       </c>
       <c r="G29" s="18" t="s">
-        <v>357</v>
+        <v>362</v>
+      </c>
+      <c r="H29" s="17" t="s">
+        <v>363</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="17" t="s">
-        <v>358</v>
+        <v>364</v>
       </c>
       <c r="B30" s="17" t="s">
-        <v>359</v>
+        <v>365</v>
       </c>
       <c r="C30" s="17" t="n">
         <v>3</v>
@@ -5061,60 +5129,69 @@
         <v>118</v>
       </c>
       <c r="F30" s="17" t="s">
-        <v>360</v>
+        <v>366</v>
       </c>
       <c r="G30" s="17"/>
+      <c r="H30" s="17"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="17" t="s">
-        <v>361</v>
+        <v>367</v>
       </c>
       <c r="B31" s="17" t="s">
-        <v>362</v>
+        <v>368</v>
       </c>
       <c r="C31" s="17" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D31" s="20" t="n">
         <f aca="false">C31*Objednávka!$C$2</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E31" s="17" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="F31" s="17" t="s">
-        <v>363</v>
-      </c>
-      <c r="G31" s="17"/>
+        <v>369</v>
+      </c>
+      <c r="G31" s="17" t="s">
+        <v>370</v>
+      </c>
+      <c r="H31" s="17" t="s">
+        <v>371</v>
+      </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="17" t="s">
-        <v>364</v>
+        <v>372</v>
       </c>
       <c r="B32" s="17" t="s">
-        <v>362</v>
+        <v>368</v>
       </c>
       <c r="C32" s="17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D32" s="20" t="n">
         <f aca="false">C32*Objednávka!$C$2</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E32" s="17" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="F32" s="17" t="s">
-        <v>365</v>
+        <v>373</v>
       </c>
       <c r="G32" s="17"/>
+      <c r="H32" s="17" t="s">
+        <v>374</v>
+      </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="17" t="s">
-        <v>366</v>
+        <v>375</v>
       </c>
       <c r="B33" s="17" t="s">
-        <v>362</v>
+        <v>368</v>
       </c>
       <c r="C33" s="17" t="n">
         <v>1</v>
@@ -5127,16 +5204,19 @@
         <v>68</v>
       </c>
       <c r="F33" s="17" t="s">
-        <v>367</v>
+        <v>376</v>
       </c>
       <c r="G33" s="17"/>
+      <c r="H33" s="17" t="s">
+        <v>377</v>
+      </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="17" t="s">
-        <v>368</v>
+        <v>378</v>
       </c>
       <c r="B34" s="17" t="s">
-        <v>369</v>
+        <v>379</v>
       </c>
       <c r="C34" s="17" t="n">
         <v>1</v>
@@ -5149,18 +5229,19 @@
         <v>142</v>
       </c>
       <c r="F34" s="17" t="s">
-        <v>370</v>
+        <v>380</v>
       </c>
       <c r="G34" s="17" t="s">
-        <v>371</v>
-      </c>
+        <v>381</v>
+      </c>
+      <c r="H34" s="17"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="17" t="s">
-        <v>372</v>
+        <v>382</v>
       </c>
       <c r="B35" s="17" t="s">
-        <v>369</v>
+        <v>379</v>
       </c>
       <c r="C35" s="17" t="n">
         <v>2</v>
@@ -5173,18 +5254,19 @@
         <v>145</v>
       </c>
       <c r="F35" s="17" t="s">
-        <v>373</v>
+        <v>383</v>
       </c>
       <c r="G35" s="17" t="s">
-        <v>374</v>
-      </c>
+        <v>384</v>
+      </c>
+      <c r="H35" s="17"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="17" t="s">
-        <v>375</v>
+        <v>385</v>
       </c>
       <c r="B36" s="17" t="s">
-        <v>376</v>
+        <v>386</v>
       </c>
       <c r="C36" s="17" t="n">
         <v>2</v>
@@ -5194,19 +5276,20 @@
         <v>2</v>
       </c>
       <c r="E36" s="17" t="s">
-        <v>377</v>
+        <v>387</v>
       </c>
       <c r="F36" s="17" t="s">
-        <v>378</v>
+        <v>388</v>
       </c>
       <c r="G36" s="17"/>
+      <c r="H36" s="17"/>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="17" t="s">
-        <v>379</v>
+        <v>389</v>
       </c>
       <c r="B37" s="17" t="s">
-        <v>376</v>
+        <v>386</v>
       </c>
       <c r="C37" s="17" t="n">
         <v>1</v>
@@ -5216,19 +5299,20 @@
         <v>1</v>
       </c>
       <c r="E37" s="17" t="s">
-        <v>380</v>
+        <v>390</v>
       </c>
       <c r="F37" s="17" t="s">
-        <v>381</v>
+        <v>391</v>
       </c>
       <c r="G37" s="17"/>
+      <c r="H37" s="17"/>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="17" t="s">
-        <v>382</v>
+        <v>392</v>
       </c>
       <c r="B38" s="17" t="s">
-        <v>376</v>
+        <v>386</v>
       </c>
       <c r="C38" s="17" t="n">
         <v>1</v>
@@ -5241,16 +5325,17 @@
         <v>130</v>
       </c>
       <c r="F38" s="17" t="s">
-        <v>383</v>
+        <v>393</v>
       </c>
       <c r="G38" s="17"/>
+      <c r="H38" s="17"/>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="17" t="s">
-        <v>384</v>
+        <v>394</v>
       </c>
       <c r="B39" s="17" t="s">
-        <v>385</v>
+        <v>395</v>
       </c>
       <c r="C39" s="17" t="n">
         <v>1</v>
@@ -5263,16 +5348,17 @@
         <v>97</v>
       </c>
       <c r="F39" s="17" t="s">
-        <v>386</v>
+        <v>396</v>
       </c>
       <c r="G39" s="17"/>
+      <c r="H39" s="17"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="17" t="s">
-        <v>387</v>
+        <v>397</v>
       </c>
       <c r="B40" s="17" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="C40" s="17" t="n">
         <v>1</v>
@@ -5285,13 +5371,14 @@
         <v>101</v>
       </c>
       <c r="F40" s="17" t="s">
-        <v>388</v>
+        <v>398</v>
       </c>
       <c r="G40" s="17"/>
+      <c r="H40" s="17"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="21" t="s">
-        <v>389</v>
+        <v>399</v>
       </c>
     </row>
   </sheetData>

</xml_diff>